<commit_message>
Commit de cambios actuales en refactor
</commit_message>
<xml_diff>
--- a/Registros/xy/angulosmediapipe/angulos0.xlsx
+++ b/Registros/xy/angulosmediapipe/angulos0.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H123"/>
+  <dimension ref="A1:H144"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -456,25 +456,25 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.178404</v>
+        <v>0.665424</v>
       </c>
       <c r="C2" t="n">
-        <v>9.037796935577893</v>
+        <v>7.508393731964889</v>
       </c>
       <c r="D2" t="n">
-        <v>8.08375233410673</v>
+        <v>12.68464350959058</v>
       </c>
       <c r="E2" t="n">
-        <v>57.32145922081447</v>
+        <v>160.2118503061649</v>
       </c>
       <c r="F2" t="n">
-        <v>127.7846108808142</v>
+        <v>168.117199910784</v>
       </c>
       <c r="G2" t="n">
-        <v>90.07363993261662</v>
+        <v>171.3600359611205</v>
       </c>
       <c r="H2" t="n">
-        <v>55.20673762037326</v>
+        <v>168.518613531042</v>
       </c>
     </row>
     <row r="3">
@@ -482,25 +482,25 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>0.239452</v>
+        <v>0.771599</v>
       </c>
       <c r="C3" t="n">
-        <v>8.820621719452282</v>
+        <v>8.47770019829669</v>
       </c>
       <c r="D3" t="n">
-        <v>8.062876933269274</v>
+        <v>12.11967827693458</v>
       </c>
       <c r="E3" t="n">
-        <v>90.52470857602964</v>
+        <v>159.7520811659087</v>
       </c>
       <c r="F3" t="n">
-        <v>154.4784714172493</v>
+        <v>169.0732150137781</v>
       </c>
       <c r="G3" t="n">
-        <v>174.3405860110774</v>
+        <v>172.6607695248444</v>
       </c>
       <c r="H3" t="n">
-        <v>146.4830654853476</v>
+        <v>169.0572037248342</v>
       </c>
     </row>
     <row r="4">
@@ -508,25 +508,25 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>0.276242</v>
+        <v>0.848712</v>
       </c>
       <c r="C4" t="n">
-        <v>9.710665033293298</v>
+        <v>9.747607791726146</v>
       </c>
       <c r="D4" t="n">
-        <v>8.672459988117017</v>
+        <v>11.98257260129148</v>
       </c>
       <c r="E4" t="n">
-        <v>134.910483738319</v>
+        <v>157.9516332923119</v>
       </c>
       <c r="F4" t="n">
-        <v>150.4716486786058</v>
+        <v>169.8220986853191</v>
       </c>
       <c r="G4" t="n">
-        <v>159.9930603803629</v>
+        <v>174.0819843457322</v>
       </c>
       <c r="H4" t="n">
-        <v>153.7584305869346</v>
+        <v>168.8007942834974</v>
       </c>
     </row>
     <row r="5">
@@ -534,25 +534,25 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>0.31688</v>
+        <v>0.921571</v>
       </c>
       <c r="C5" t="n">
-        <v>9.945999335181837</v>
+        <v>10.01758196559489</v>
       </c>
       <c r="D5" t="n">
-        <v>8.851620575722027</v>
+        <v>11.48040365123644</v>
       </c>
       <c r="E5" t="n">
-        <v>121.4545570377371</v>
+        <v>157.3363995493422</v>
       </c>
       <c r="F5" t="n">
-        <v>151.2495605118422</v>
+        <v>170.4473730693543</v>
       </c>
       <c r="G5" t="n">
-        <v>162.1632726625836</v>
+        <v>174.0949862870312</v>
       </c>
       <c r="H5" t="n">
-        <v>152.4849337422978</v>
+        <v>169.0571651711999</v>
       </c>
     </row>
     <row r="6">
@@ -560,25 +560,25 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>0.354358</v>
+        <v>0.989888</v>
       </c>
       <c r="C6" t="n">
-        <v>10.26486270676991</v>
+        <v>10.05044849752987</v>
       </c>
       <c r="D6" t="n">
-        <v>8.993443429336056</v>
+        <v>11.35305421576956</v>
       </c>
       <c r="E6" t="n">
-        <v>144.6774959468495</v>
+        <v>157.1960912249472</v>
       </c>
       <c r="F6" t="n">
-        <v>152.0742865161551</v>
+        <v>170.5678383279057</v>
       </c>
       <c r="G6" t="n">
-        <v>164.1848439951224</v>
+        <v>173.980860829621</v>
       </c>
       <c r="H6" t="n">
-        <v>170.2387093610516</v>
+        <v>169.0693676294987</v>
       </c>
     </row>
     <row r="7">
@@ -586,25 +586,25 @@
         <v>5</v>
       </c>
       <c r="B7" t="n">
-        <v>0.39014</v>
+        <v>1.052202</v>
       </c>
       <c r="C7" t="n">
-        <v>10.20960114916646</v>
+        <v>10.080918459925</v>
       </c>
       <c r="D7" t="n">
-        <v>9.100616222086149</v>
+        <v>11.25177027552821</v>
       </c>
       <c r="E7" t="n">
-        <v>155.8761133073986</v>
+        <v>157.8878981982515</v>
       </c>
       <c r="F7" t="n">
-        <v>148.2252376688797</v>
+        <v>170.7308090359884</v>
       </c>
       <c r="G7" t="n">
-        <v>154.6334037103614</v>
+        <v>173.9598178935781</v>
       </c>
       <c r="H7" t="n">
-        <v>174.5154347988698</v>
+        <v>168.5234112439607</v>
       </c>
     </row>
     <row r="8">
@@ -612,25 +612,25 @@
         <v>6</v>
       </c>
       <c r="B8" t="n">
-        <v>0.428012</v>
+        <v>1.122077</v>
       </c>
       <c r="C8" t="n">
-        <v>11.64786385379155</v>
+        <v>9.936024387570876</v>
       </c>
       <c r="D8" t="n">
-        <v>9.098868252612396</v>
+        <v>11.36664307695056</v>
       </c>
       <c r="E8" t="n">
-        <v>159.8986440402672</v>
+        <v>158.2281165985257</v>
       </c>
       <c r="F8" t="n">
-        <v>152.8412961670004</v>
+        <v>172.1023972410093</v>
       </c>
       <c r="G8" t="n">
-        <v>160.4904478873532</v>
+        <v>169.8102742042887</v>
       </c>
       <c r="H8" t="n">
-        <v>174.7592914116047</v>
+        <v>168.0946877702985</v>
       </c>
     </row>
     <row r="9">
@@ -638,25 +638,25 @@
         <v>7</v>
       </c>
       <c r="B9" t="n">
-        <v>0.468868</v>
+        <v>1.190593</v>
       </c>
       <c r="C9" t="n">
-        <v>11.48679378971795</v>
+        <v>9.83645781852395</v>
       </c>
       <c r="D9" t="n">
-        <v>9.150766421394696</v>
+        <v>11.33739354076311</v>
       </c>
       <c r="E9" t="n">
-        <v>155.7055310567427</v>
+        <v>158.3247255232507</v>
       </c>
       <c r="F9" t="n">
-        <v>152.7366091739042</v>
+        <v>172.8113760622518</v>
       </c>
       <c r="G9" t="n">
-        <v>159.5187055167692</v>
+        <v>168.3145288299047</v>
       </c>
       <c r="H9" t="n">
-        <v>177.3222282266452</v>
+        <v>168.0908961954044</v>
       </c>
     </row>
     <row r="10">
@@ -664,25 +664,25 @@
         <v>8</v>
       </c>
       <c r="B10" t="n">
-        <v>0.506537</v>
+        <v>1.250939</v>
       </c>
       <c r="C10" t="n">
-        <v>11.01676993630447</v>
+        <v>10.12323818561293</v>
       </c>
       <c r="D10" t="n">
-        <v>9.577623478569327</v>
+        <v>11.56847291382433</v>
       </c>
       <c r="E10" t="n">
-        <v>158.5956085517936</v>
+        <v>157.9245653609179</v>
       </c>
       <c r="F10" t="n">
-        <v>152.828417432613</v>
+        <v>172.95759253258</v>
       </c>
       <c r="G10" t="n">
-        <v>159.4250140021426</v>
+        <v>169.5950083836703</v>
       </c>
       <c r="H10" t="n">
-        <v>177.4826851758005</v>
+        <v>167.8814392910193</v>
       </c>
     </row>
     <row r="11">
@@ -690,25 +690,25 @@
         <v>9</v>
       </c>
       <c r="B11" t="n">
-        <v>0.5454639999999999</v>
+        <v>1.321022</v>
       </c>
       <c r="C11" t="n">
-        <v>10.85916766604652</v>
+        <v>9.976588720949405</v>
       </c>
       <c r="D11" t="n">
-        <v>9.868629015699023</v>
+        <v>11.58747294733882</v>
       </c>
       <c r="E11" t="n">
-        <v>160.9642607894902</v>
+        <v>157.8750967781017</v>
       </c>
       <c r="F11" t="n">
-        <v>151.8730769041657</v>
+        <v>172.8922600116648</v>
       </c>
       <c r="G11" t="n">
-        <v>156.6736480992183</v>
+        <v>171.3948307112883</v>
       </c>
       <c r="H11" t="n">
-        <v>177.1828390233974</v>
+        <v>167.823039333737</v>
       </c>
     </row>
     <row r="12">
@@ -716,25 +716,25 @@
         <v>10</v>
       </c>
       <c r="B12" t="n">
-        <v>0.585537</v>
+        <v>1.383644</v>
       </c>
       <c r="C12" t="n">
-        <v>10.85225381035319</v>
+        <v>9.968417344470028</v>
       </c>
       <c r="D12" t="n">
-        <v>9.394001399350669</v>
+        <v>11.61854518632089</v>
       </c>
       <c r="E12" t="n">
-        <v>155.1847318382864</v>
+        <v>157.6248256797022</v>
       </c>
       <c r="F12" t="n">
-        <v>152.8822661034096</v>
+        <v>172.8400058127892</v>
       </c>
       <c r="G12" t="n">
-        <v>158.1439179680524</v>
+        <v>172.0398589873799</v>
       </c>
       <c r="H12" t="n">
-        <v>135.6019301922503</v>
+        <v>167.8663885520953</v>
       </c>
     </row>
     <row r="13">
@@ -742,25 +742,25 @@
         <v>11</v>
       </c>
       <c r="B13" t="n">
-        <v>0.620586</v>
+        <v>1.441278</v>
       </c>
       <c r="C13" t="n">
-        <v>9.79949223721264</v>
+        <v>9.887824490758687</v>
       </c>
       <c r="D13" t="n">
-        <v>9.4936226944008</v>
+        <v>11.7115598332192</v>
       </c>
       <c r="E13" t="n">
-        <v>144.6785751582039</v>
+        <v>157.6613193279795</v>
       </c>
       <c r="F13" t="n">
-        <v>152.5341869129083</v>
+        <v>172.8497814238562</v>
       </c>
       <c r="G13" t="n">
-        <v>158.004296825102</v>
+        <v>171.8458245085789</v>
       </c>
       <c r="H13" t="n">
-        <v>115.4470952932306</v>
+        <v>167.9943754586257</v>
       </c>
     </row>
     <row r="14">
@@ -768,25 +768,25 @@
         <v>12</v>
       </c>
       <c r="B14" t="n">
-        <v>0.658048</v>
+        <v>1.511314</v>
       </c>
       <c r="C14" t="n">
-        <v>10.06837280768846</v>
+        <v>9.905254102649343</v>
       </c>
       <c r="D14" t="n">
-        <v>9.526074621056891</v>
+        <v>11.67237084728416</v>
       </c>
       <c r="E14" t="n">
-        <v>157.0907507061679</v>
+        <v>157.8594298773154</v>
       </c>
       <c r="F14" t="n">
-        <v>153.4145946565223</v>
+        <v>172.7212734613849</v>
       </c>
       <c r="G14" t="n">
-        <v>161.0093491054799</v>
+        <v>171.3830578668243</v>
       </c>
       <c r="H14" t="n">
-        <v>172.793108209238</v>
+        <v>168.2494462528414</v>
       </c>
     </row>
     <row r="15">
@@ -794,25 +794,25 @@
         <v>13</v>
       </c>
       <c r="B15" t="n">
-        <v>0.695612</v>
+        <v>1.584471</v>
       </c>
       <c r="C15" t="n">
-        <v>9.972369883302953</v>
+        <v>9.981856069120019</v>
       </c>
       <c r="D15" t="n">
-        <v>9.859827348101316</v>
+        <v>11.62235344474684</v>
       </c>
       <c r="E15" t="n">
-        <v>155.7956099358539</v>
+        <v>157.9288272120478</v>
       </c>
       <c r="F15" t="n">
-        <v>152.4482719381385</v>
+        <v>172.5866612412264</v>
       </c>
       <c r="G15" t="n">
-        <v>159.599725435319</v>
+        <v>170.7657961857437</v>
       </c>
       <c r="H15" t="n">
-        <v>170.5171635614175</v>
+        <v>168.3248852916186</v>
       </c>
     </row>
     <row r="16">
@@ -820,25 +820,25 @@
         <v>14</v>
       </c>
       <c r="B16" t="n">
-        <v>0.740109</v>
+        <v>1.648771</v>
       </c>
       <c r="C16" t="n">
-        <v>9.820222375401963</v>
+        <v>9.963233996722265</v>
       </c>
       <c r="D16" t="n">
-        <v>9.918764758466116</v>
+        <v>11.78508664169529</v>
       </c>
       <c r="E16" t="n">
-        <v>157.1272698361063</v>
+        <v>157.9930467572459</v>
       </c>
       <c r="F16" t="n">
-        <v>154.6012445857867</v>
+        <v>172.4387011111223</v>
       </c>
       <c r="G16" t="n">
-        <v>163.9715806599732</v>
+        <v>169.5801031472672</v>
       </c>
       <c r="H16" t="n">
-        <v>174.1690834749377</v>
+        <v>168.226616504757</v>
       </c>
     </row>
     <row r="17">
@@ -846,25 +846,25 @@
         <v>15</v>
       </c>
       <c r="B17" t="n">
-        <v>0.779007</v>
+        <v>1.719999</v>
       </c>
       <c r="C17" t="n">
-        <v>9.923373131318549</v>
+        <v>10.36233738989721</v>
       </c>
       <c r="D17" t="n">
-        <v>10.03484709809579</v>
+        <v>11.85658515451175</v>
       </c>
       <c r="E17" t="n">
-        <v>158.5317970498806</v>
+        <v>156.8392107811327</v>
       </c>
       <c r="F17" t="n">
-        <v>153.6153091599816</v>
+        <v>171.9262282266234</v>
       </c>
       <c r="G17" t="n">
-        <v>162.2253414300258</v>
+        <v>169.8944775904514</v>
       </c>
       <c r="H17" t="n">
-        <v>174.2109037385463</v>
+        <v>168.0922775278587</v>
       </c>
     </row>
     <row r="18">
@@ -872,25 +872,25 @@
         <v>16</v>
       </c>
       <c r="B18" t="n">
-        <v>0.819078</v>
+        <v>1.786078</v>
       </c>
       <c r="C18" t="n">
-        <v>9.886748675743103</v>
+        <v>10.57312410370606</v>
       </c>
       <c r="D18" t="n">
-        <v>10.12788480034067</v>
+        <v>11.92948769500307</v>
       </c>
       <c r="E18" t="n">
-        <v>161.6914062971875</v>
+        <v>156.2428431849345</v>
       </c>
       <c r="F18" t="n">
-        <v>155.1045156778719</v>
+        <v>171.5521904533539</v>
       </c>
       <c r="G18" t="n">
-        <v>163.6745366156433</v>
+        <v>170.2308419601312</v>
       </c>
       <c r="H18" t="n">
-        <v>175.1224966023965</v>
+        <v>168.1199375913142</v>
       </c>
     </row>
     <row r="19">
@@ -898,25 +898,25 @@
         <v>17</v>
       </c>
       <c r="B19" t="n">
-        <v>0.861697</v>
+        <v>1.852061</v>
       </c>
       <c r="C19" t="n">
-        <v>8.975909118334529</v>
+        <v>10.02654677523358</v>
       </c>
       <c r="D19" t="n">
-        <v>10.16463594523857</v>
+        <v>11.94093681943119</v>
       </c>
       <c r="E19" t="n">
-        <v>161.9540808553316</v>
+        <v>157.6897993790654</v>
       </c>
       <c r="F19" t="n">
-        <v>148.5871446804846</v>
+        <v>171.7184693202738</v>
       </c>
       <c r="G19" t="n">
-        <v>152.1951172981066</v>
+        <v>170.3031223881368</v>
       </c>
       <c r="H19" t="n">
-        <v>173.8265833267425</v>
+        <v>167.5565993619483</v>
       </c>
     </row>
     <row r="20">
@@ -924,25 +924,25 @@
         <v>18</v>
       </c>
       <c r="B20" t="n">
-        <v>0.8962560000000001</v>
+        <v>1.910373</v>
       </c>
       <c r="C20" t="n">
-        <v>9.027781007241986</v>
+        <v>10.28878445392136</v>
       </c>
       <c r="D20" t="n">
-        <v>10.14387236458627</v>
+        <v>12.04209554672557</v>
       </c>
       <c r="E20" t="n">
-        <v>161.0827449726875</v>
+        <v>158.9574497674403</v>
       </c>
       <c r="F20" t="n">
-        <v>147.955855541859</v>
+        <v>171.5138096774611</v>
       </c>
       <c r="G20" t="n">
-        <v>154.6373741482631</v>
+        <v>170.4321193127728</v>
       </c>
       <c r="H20" t="n">
-        <v>169.9836591248032</v>
+        <v>167.1501627537982</v>
       </c>
     </row>
     <row r="21">
@@ -950,25 +950,25 @@
         <v>19</v>
       </c>
       <c r="B21" t="n">
-        <v>0.937329</v>
+        <v>1.97809</v>
       </c>
       <c r="C21" t="n">
-        <v>9.04772511269238</v>
+        <v>10.4650783045454</v>
       </c>
       <c r="D21" t="n">
-        <v>10.26649675478797</v>
+        <v>12.10124511804452</v>
       </c>
       <c r="E21" t="n">
-        <v>156.3825893818041</v>
+        <v>159.2958046272575</v>
       </c>
       <c r="F21" t="n">
-        <v>147.5098127027236</v>
+        <v>171.3938018856739</v>
       </c>
       <c r="G21" t="n">
-        <v>154.4383171215582</v>
+        <v>170.5055673886345</v>
       </c>
       <c r="H21" t="n">
-        <v>153.6920739554944</v>
+        <v>166.8717487226969</v>
       </c>
     </row>
     <row r="22">
@@ -976,25 +976,25 @@
         <v>20</v>
       </c>
       <c r="B22" t="n">
-        <v>0.976471</v>
+        <v>2.033657</v>
       </c>
       <c r="C22" t="n">
-        <v>9.430580533700677</v>
+        <v>10.50009191948281</v>
       </c>
       <c r="D22" t="n">
-        <v>11.02947574115469</v>
+        <v>11.91427121400257</v>
       </c>
       <c r="E22" t="n">
-        <v>148.0100394062536</v>
+        <v>159.9881680852304</v>
       </c>
       <c r="F22" t="n">
-        <v>147.4226176963616</v>
+        <v>171.5082265951302</v>
       </c>
       <c r="G22" t="n">
-        <v>157.2791164688022</v>
+        <v>170.8840451391767</v>
       </c>
       <c r="H22" t="n">
-        <v>140.5850415055571</v>
+        <v>168.6437269754854</v>
       </c>
     </row>
     <row r="23">
@@ -1002,25 +1002,25 @@
         <v>21</v>
       </c>
       <c r="B23" t="n">
-        <v>1.016226</v>
+        <v>2.106141</v>
       </c>
       <c r="C23" t="n">
-        <v>9.326326580745807</v>
+        <v>10.64782736310835</v>
       </c>
       <c r="D23" t="n">
-        <v>10.86825161709817</v>
+        <v>11.67740124365549</v>
       </c>
       <c r="E23" t="n">
-        <v>154.6561980499458</v>
+        <v>160.3168714295528</v>
       </c>
       <c r="F23" t="n">
-        <v>151.1970264159684</v>
+        <v>171.9603847241639</v>
       </c>
       <c r="G23" t="n">
-        <v>161.7815155491146</v>
+        <v>170.0355647542602</v>
       </c>
       <c r="H23" t="n">
-        <v>168.4146423861322</v>
+        <v>168.5621135047369</v>
       </c>
     </row>
     <row r="24">
@@ -1028,25 +1028,25 @@
         <v>22</v>
       </c>
       <c r="B24" t="n">
-        <v>1.053409</v>
+        <v>2.178536</v>
       </c>
       <c r="C24" t="n">
-        <v>10.31524408951422</v>
+        <v>10.75551587036645</v>
       </c>
       <c r="D24" t="n">
-        <v>10.708476092896</v>
+        <v>11.5497195594329</v>
       </c>
       <c r="E24" t="n">
-        <v>151.1271114135772</v>
+        <v>160.4536742826801</v>
       </c>
       <c r="F24" t="n">
-        <v>153.7744473945116</v>
+        <v>172.1926172241926</v>
       </c>
       <c r="G24" t="n">
-        <v>164.5722794738673</v>
+        <v>169.5986628873911</v>
       </c>
       <c r="H24" t="n">
-        <v>166.2584449917998</v>
+        <v>168.4793994680235</v>
       </c>
     </row>
     <row r="25">
@@ -1054,25 +1054,25 @@
         <v>23</v>
       </c>
       <c r="B25" t="n">
-        <v>1.095251</v>
+        <v>2.247167</v>
       </c>
       <c r="C25" t="n">
-        <v>10.67683800515634</v>
+        <v>12.38898598454429</v>
       </c>
       <c r="D25" t="n">
-        <v>10.43158197313515</v>
+        <v>14.44201188519331</v>
       </c>
       <c r="E25" t="n">
-        <v>155.7701989559083</v>
+        <v>157.3142046013635</v>
       </c>
       <c r="F25" t="n">
-        <v>159.2243699288301</v>
+        <v>171.6685662490192</v>
       </c>
       <c r="G25" t="n">
-        <v>165.8987552921714</v>
+        <v>167.2812725788057</v>
       </c>
       <c r="H25" t="n">
-        <v>170.8927346931625</v>
+        <v>167.4117085815579</v>
       </c>
     </row>
     <row r="26">
@@ -1080,25 +1080,25 @@
         <v>24</v>
       </c>
       <c r="B26" t="n">
-        <v>1.131318</v>
+        <v>2.314051</v>
       </c>
       <c r="C26" t="n">
-        <v>11.83975701821592</v>
+        <v>14.29748634958397</v>
       </c>
       <c r="D26" t="n">
-        <v>10.59522222049344</v>
+        <v>20.65968487043876</v>
       </c>
       <c r="E26" t="n">
-        <v>154.6550269237388</v>
+        <v>158.9422542349959</v>
       </c>
       <c r="F26" t="n">
-        <v>157.967034666939</v>
+        <v>177.1901413326519</v>
       </c>
       <c r="G26" t="n">
-        <v>165.004549718106</v>
+        <v>163.1072094547984</v>
       </c>
       <c r="H26" t="n">
-        <v>168.7958911317454</v>
+        <v>166.6372697060407</v>
       </c>
     </row>
     <row r="27">
@@ -1106,25 +1106,25 @@
         <v>25</v>
       </c>
       <c r="B27" t="n">
-        <v>1.166312</v>
+        <v>2.386655</v>
       </c>
       <c r="C27" t="n">
-        <v>12.17571441410121</v>
+        <v>15.12295604454192</v>
       </c>
       <c r="D27" t="n">
-        <v>10.81490122882658</v>
+        <v>22.62091234709263</v>
       </c>
       <c r="E27" t="n">
-        <v>155.0322495464366</v>
+        <v>159.0604977164192</v>
       </c>
       <c r="F27" t="n">
-        <v>159.4099140107617</v>
+        <v>176.1682164528644</v>
       </c>
       <c r="G27" t="n">
-        <v>159.3705949499561</v>
+        <v>162.9954331690327</v>
       </c>
       <c r="H27" t="n">
-        <v>170.3295212031117</v>
+        <v>166.5907545319563</v>
       </c>
     </row>
     <row r="28">
@@ -1132,25 +1132,25 @@
         <v>26</v>
       </c>
       <c r="B28" t="n">
-        <v>1.202044</v>
+        <v>2.441616</v>
       </c>
       <c r="C28" t="n">
-        <v>12.1890693312679</v>
+        <v>14.4409334746421</v>
       </c>
       <c r="D28" t="n">
-        <v>11.45638844910104</v>
+        <v>27.69172707298049</v>
       </c>
       <c r="E28" t="n">
-        <v>154.5807720609323</v>
+        <v>159.0018782826965</v>
       </c>
       <c r="F28" t="n">
-        <v>157.5959927430702</v>
+        <v>114.8035692799901</v>
       </c>
       <c r="G28" t="n">
-        <v>160.7749003323102</v>
+        <v>109.4446558902812</v>
       </c>
       <c r="H28" t="n">
-        <v>169.1553225167323</v>
+        <v>168.5838391784704</v>
       </c>
     </row>
     <row r="29">
@@ -1158,25 +1158,25 @@
         <v>27</v>
       </c>
       <c r="B29" t="n">
-        <v>1.236654</v>
+        <v>2.501961</v>
       </c>
       <c r="C29" t="n">
-        <v>12.52321000086968</v>
+        <v>14.59530808322853</v>
       </c>
       <c r="D29" t="n">
-        <v>12.6143446754534</v>
+        <v>36.28810470521908</v>
       </c>
       <c r="E29" t="n">
-        <v>131.8806498919406</v>
+        <v>162.0901450638551</v>
       </c>
       <c r="F29" t="n">
-        <v>27.06902437741751</v>
+        <v>86.4712648030128</v>
       </c>
       <c r="G29" t="n">
-        <v>164.9553314898425</v>
+        <v>135.7324122750461</v>
       </c>
       <c r="H29" t="n">
-        <v>141.4646838335199</v>
+        <v>165.9390596325272</v>
       </c>
     </row>
     <row r="30">
@@ -1184,25 +1184,25 @@
         <v>28</v>
       </c>
       <c r="B30" t="n">
-        <v>1.284158</v>
+        <v>2.569601</v>
       </c>
       <c r="C30" t="n">
-        <v>12.69423634011866</v>
+        <v>15.08605948756111</v>
       </c>
       <c r="D30" t="n">
-        <v>13.28303223959558</v>
+        <v>38.38775843868627</v>
       </c>
       <c r="E30" t="n">
-        <v>64.68168051705509</v>
+        <v>160.3072256962305</v>
       </c>
       <c r="F30" t="n">
-        <v>19.50976060391053</v>
+        <v>84.34199029903807</v>
       </c>
       <c r="G30" t="n">
-        <v>158.6246567899151</v>
+        <v>138.5459331168615</v>
       </c>
       <c r="H30" t="n">
-        <v>138.986807609905</v>
+        <v>170.4313520847703</v>
       </c>
     </row>
     <row r="31">
@@ -1210,25 +1210,25 @@
         <v>29</v>
       </c>
       <c r="B31" t="n">
-        <v>1.322265</v>
+        <v>2.632045</v>
       </c>
       <c r="C31" t="n">
-        <v>12.87037377100617</v>
+        <v>17.20505977036674</v>
       </c>
       <c r="D31" t="n">
-        <v>11.87975778747771</v>
+        <v>50.19327295263347</v>
       </c>
       <c r="E31" t="n">
-        <v>89.58934466677948</v>
+        <v>162.1334249444746</v>
       </c>
       <c r="F31" t="n">
-        <v>20.98621575541711</v>
+        <v>67.05520624509228</v>
       </c>
       <c r="G31" t="n">
-        <v>153.1184019990741</v>
+        <v>159.9746135368534</v>
       </c>
       <c r="H31" t="n">
-        <v>142.0824793363681</v>
+        <v>165.0599446262511</v>
       </c>
     </row>
     <row r="32">
@@ -1236,25 +1236,25 @@
         <v>30</v>
       </c>
       <c r="B32" t="n">
-        <v>1.360993</v>
+        <v>2.704404</v>
       </c>
       <c r="C32" t="n">
-        <v>12.89857482366927</v>
+        <v>19.04623430559601</v>
       </c>
       <c r="D32" t="n">
-        <v>10.95372562512287</v>
+        <v>57.82391478611113</v>
       </c>
       <c r="E32" t="n">
-        <v>76.59255852123121</v>
+        <v>164.2942529566146</v>
       </c>
       <c r="F32" t="n">
-        <v>23.18006889698738</v>
+        <v>68.389541848967</v>
       </c>
       <c r="G32" t="n">
-        <v>150.521545379991</v>
+        <v>165.8219859429128</v>
       </c>
       <c r="H32" t="n">
-        <v>137.7513091822082</v>
+        <v>163.7259659747703</v>
       </c>
     </row>
     <row r="33">
@@ -1262,25 +1262,25 @@
         <v>31</v>
       </c>
       <c r="B33" t="n">
-        <v>1.401322</v>
+        <v>2.766391</v>
       </c>
       <c r="C33" t="n">
-        <v>10.22473047731331</v>
+        <v>24.52400486728389</v>
       </c>
       <c r="D33" t="n">
-        <v>10.45808054049364</v>
+        <v>58.37489747409537</v>
       </c>
       <c r="E33" t="n">
-        <v>27.281046051728</v>
+        <v>159.4920931681112</v>
       </c>
       <c r="F33" t="n">
-        <v>16.59074444242208</v>
+        <v>68.2685195364714</v>
       </c>
       <c r="G33" t="n">
-        <v>165.8693246048295</v>
+        <v>166.8565566590268</v>
       </c>
       <c r="H33" t="n">
-        <v>161.2792036673368</v>
+        <v>162.1364004778159</v>
       </c>
     </row>
     <row r="34">
@@ -1288,25 +1288,25 @@
         <v>32</v>
       </c>
       <c r="B34" t="n">
-        <v>1.439332</v>
+        <v>2.828114</v>
       </c>
       <c r="C34" t="n">
-        <v>10.21972057217402</v>
+        <v>26.99315559771347</v>
       </c>
       <c r="D34" t="n">
-        <v>8.69257436204275</v>
+        <v>62.93503220225468</v>
       </c>
       <c r="E34" t="n">
-        <v>28.56939058185437</v>
+        <v>160.1983062665262</v>
       </c>
       <c r="F34" t="n">
-        <v>18.99770441317402</v>
+        <v>64.87898978917303</v>
       </c>
       <c r="G34" t="n">
-        <v>160.3857525150969</v>
+        <v>175.3874062842246</v>
       </c>
       <c r="H34" t="n">
-        <v>131.9617683777952</v>
+        <v>164.2765122787809</v>
       </c>
     </row>
     <row r="35">
@@ -1314,25 +1314,25 @@
         <v>33</v>
       </c>
       <c r="B35" t="n">
-        <v>1.481829</v>
+        <v>2.893976</v>
       </c>
       <c r="C35" t="n">
-        <v>9.197135274740914</v>
+        <v>26.54374602077533</v>
       </c>
       <c r="D35" t="n">
-        <v>9.044032843279265</v>
+        <v>66.64789459025629</v>
       </c>
       <c r="E35" t="n">
-        <v>26.0621182111984</v>
+        <v>155.2778015082048</v>
       </c>
       <c r="F35" t="n">
-        <v>16.24702520269623</v>
+        <v>65.04487701582755</v>
       </c>
       <c r="G35" t="n">
-        <v>172.4624429403752</v>
+        <v>174.2809358085663</v>
       </c>
       <c r="H35" t="n">
-        <v>121.5887984899004</v>
+        <v>164.5201708558061</v>
       </c>
     </row>
     <row r="36">
@@ -1340,25 +1340,25 @@
         <v>34</v>
       </c>
       <c r="B36" t="n">
-        <v>1.518402</v>
+        <v>2.964396</v>
       </c>
       <c r="C36" t="n">
-        <v>7.114612728976372</v>
+        <v>24.7221270922248</v>
       </c>
       <c r="D36" t="n">
-        <v>9.454007814073188</v>
+        <v>66.93159262590893</v>
       </c>
       <c r="E36" t="n">
-        <v>25.9765587546168</v>
+        <v>155.0854540674034</v>
       </c>
       <c r="F36" t="n">
-        <v>18.10999490683746</v>
+        <v>64.58891007239025</v>
       </c>
       <c r="G36" t="n">
-        <v>174.1627025138433</v>
+        <v>174.3243001667118</v>
       </c>
       <c r="H36" t="n">
-        <v>156.62549350667</v>
+        <v>163.8122596453791</v>
       </c>
     </row>
     <row r="37">
@@ -1366,25 +1366,25 @@
         <v>35</v>
       </c>
       <c r="B37" t="n">
-        <v>1.55355</v>
+        <v>3.0313</v>
       </c>
       <c r="C37" t="n">
-        <v>4.989203059284838</v>
+        <v>66.37606892334027</v>
       </c>
       <c r="D37" t="n">
-        <v>9.6319642544349</v>
+        <v>68.8938983421166</v>
       </c>
       <c r="E37" t="n">
-        <v>25.23672493165493</v>
+        <v>51.65713275308208</v>
       </c>
       <c r="F37" t="n">
-        <v>23.13376957517922</v>
+        <v>55.96918500497031</v>
       </c>
       <c r="G37" t="n">
-        <v>162.5158884355553</v>
+        <v>178.1825456722406</v>
       </c>
       <c r="H37" t="n">
-        <v>169.403847500234</v>
+        <v>174.964412605296</v>
       </c>
     </row>
     <row r="38">
@@ -1392,25 +1392,25 @@
         <v>36</v>
       </c>
       <c r="B38" t="n">
-        <v>1.591644</v>
+        <v>3.100301</v>
       </c>
       <c r="C38" t="n">
-        <v>5.076461148803793</v>
+        <v>57.57981527847437</v>
       </c>
       <c r="D38" t="n">
-        <v>9.032244807006697</v>
+        <v>69.46383596601888</v>
       </c>
       <c r="E38" t="n">
-        <v>26.16304555932669</v>
+        <v>42.82777823593672</v>
       </c>
       <c r="F38" t="n">
-        <v>23.32588688862401</v>
+        <v>50.27238827731424</v>
       </c>
       <c r="G38" t="n">
-        <v>164.5204194157365</v>
+        <v>176.462411401979</v>
       </c>
       <c r="H38" t="n">
-        <v>164.2959370640701</v>
+        <v>179.2899378692464</v>
       </c>
     </row>
     <row r="39">
@@ -1418,25 +1418,25 @@
         <v>37</v>
       </c>
       <c r="B39" t="n">
-        <v>1.628195</v>
+        <v>3.169173</v>
       </c>
       <c r="C39" t="n">
-        <v>4.985260671115834</v>
+        <v>57.08794203197638</v>
       </c>
       <c r="D39" t="n">
-        <v>8.661924110755077</v>
+        <v>69.4024554155812</v>
       </c>
       <c r="E39" t="n">
-        <v>25.10962028831851</v>
+        <v>42.05108263966387</v>
       </c>
       <c r="F39" t="n">
-        <v>22.43943318587898</v>
+        <v>48.73489091472808</v>
       </c>
       <c r="G39" t="n">
-        <v>164.5979487619041</v>
+        <v>174.3534389724077</v>
       </c>
       <c r="H39" t="n">
-        <v>166.9582779935001</v>
+        <v>175.5176256904275</v>
       </c>
     </row>
     <row r="40">
@@ -1444,25 +1444,25 @@
         <v>38</v>
       </c>
       <c r="B40" t="n">
-        <v>1.665009</v>
+        <v>3.228742</v>
       </c>
       <c r="C40" t="n">
-        <v>4.491367066754957</v>
+        <v>57.26895845134366</v>
       </c>
       <c r="D40" t="n">
-        <v>8.298118244903328</v>
+        <v>72.50474919275774</v>
       </c>
       <c r="E40" t="n">
-        <v>25.29575801509084</v>
+        <v>39.46722285140497</v>
       </c>
       <c r="F40" t="n">
-        <v>21.60442434540781</v>
+        <v>45.6902911670454</v>
       </c>
       <c r="G40" t="n">
-        <v>165.1427271401681</v>
+        <v>173.7457726562014</v>
       </c>
       <c r="H40" t="n">
-        <v>167.2225654078303</v>
+        <v>173.786522427587</v>
       </c>
     </row>
     <row r="41">
@@ -1470,25 +1470,25 @@
         <v>39</v>
       </c>
       <c r="B41" t="n">
-        <v>1.699123</v>
+        <v>3.290992</v>
       </c>
       <c r="C41" t="n">
-        <v>5.743706664883528</v>
+        <v>57.84116593376354</v>
       </c>
       <c r="D41" t="n">
-        <v>7.931166301631677</v>
+        <v>74.05501561883976</v>
       </c>
       <c r="E41" t="n">
-        <v>23.80642210910199</v>
+        <v>42.38460399314689</v>
       </c>
       <c r="F41" t="n">
-        <v>19.30547707727227</v>
+        <v>44.74738816925132</v>
       </c>
       <c r="G41" t="n">
-        <v>167.4828668828631</v>
+        <v>174.0328635825765</v>
       </c>
       <c r="H41" t="n">
-        <v>166.537443546944</v>
+        <v>161.0872018703871</v>
       </c>
     </row>
     <row r="42">
@@ -1496,25 +1496,25 @@
         <v>40</v>
       </c>
       <c r="B42" t="n">
-        <v>1.733472</v>
+        <v>3.36076</v>
       </c>
       <c r="C42" t="n">
-        <v>9.936483600757867</v>
+        <v>61.33380549617804</v>
       </c>
       <c r="D42" t="n">
-        <v>7.659307225051522</v>
+        <v>74.85414731376497</v>
       </c>
       <c r="E42" t="n">
-        <v>10.52953049355036</v>
+        <v>44.89510308164157</v>
       </c>
       <c r="F42" t="n">
-        <v>18.98525453670186</v>
+        <v>44.42438357546739</v>
       </c>
       <c r="G42" t="n">
-        <v>169.3836210398797</v>
+        <v>172.0836805335206</v>
       </c>
       <c r="H42" t="n">
-        <v>170.6648455848752</v>
+        <v>158.9488953397441</v>
       </c>
     </row>
     <row r="43">
@@ -1522,25 +1522,25 @@
         <v>41</v>
       </c>
       <c r="B43" t="n">
-        <v>1.768337</v>
+        <v>3.429156</v>
       </c>
       <c r="C43" t="n">
-        <v>13.97709416334901</v>
+        <v>57.37869216307939</v>
       </c>
       <c r="D43" t="n">
-        <v>8.007096264180335</v>
+        <v>78.51958647091075</v>
       </c>
       <c r="E43" t="n">
-        <v>159.7080472720135</v>
+        <v>37.44454662199879</v>
       </c>
       <c r="F43" t="n">
-        <v>18.60260209888035</v>
+        <v>44.36335201648649</v>
       </c>
       <c r="G43" t="n">
-        <v>171.0502502720316</v>
+        <v>174.6649854984672</v>
       </c>
       <c r="H43" t="n">
-        <v>155.4804431723464</v>
+        <v>170.1448008029788</v>
       </c>
     </row>
     <row r="44">
@@ -1548,25 +1548,25 @@
         <v>42</v>
       </c>
       <c r="B44" t="n">
-        <v>1.802434</v>
+        <v>3.498539</v>
       </c>
       <c r="C44" t="n">
-        <v>17.27662882861624</v>
+        <v>54.8567195455713</v>
       </c>
       <c r="D44" t="n">
-        <v>9.363648002211644</v>
+        <v>82.29362831614051</v>
       </c>
       <c r="E44" t="n">
-        <v>155.9075713079791</v>
+        <v>34.23038013610163</v>
       </c>
       <c r="F44" t="n">
-        <v>15.86094673402105</v>
+        <v>45.95597398093318</v>
       </c>
       <c r="G44" t="n">
-        <v>177.5246907998145</v>
+        <v>178.963972416463</v>
       </c>
       <c r="H44" t="n">
-        <v>41.53177978578736</v>
+        <v>174.3424825369634</v>
       </c>
     </row>
     <row r="45">
@@ -1574,25 +1574,25 @@
         <v>43</v>
       </c>
       <c r="B45" t="n">
-        <v>1.835961</v>
+        <v>3.567509</v>
       </c>
       <c r="C45" t="n">
-        <v>21.76550926022999</v>
+        <v>53.45636055000984</v>
       </c>
       <c r="D45" t="n">
-        <v>10.29394571202866</v>
+        <v>82.92481930894604</v>
       </c>
       <c r="E45" t="n">
-        <v>116.765231759989</v>
+        <v>33.07879318862254</v>
       </c>
       <c r="F45" t="n">
-        <v>15.35500136886366</v>
+        <v>46.23002554381288</v>
       </c>
       <c r="G45" t="n">
-        <v>176.5104446375159</v>
+        <v>179.6053607534041</v>
       </c>
       <c r="H45" t="n">
-        <v>108.9339059137861</v>
+        <v>175.1113412564324</v>
       </c>
     </row>
     <row r="46">
@@ -1600,25 +1600,25 @@
         <v>44</v>
       </c>
       <c r="B46" t="n">
-        <v>1.869765</v>
+        <v>3.636462</v>
       </c>
       <c r="C46" t="n">
-        <v>20.55770154859406</v>
+        <v>52.86723858078997</v>
       </c>
       <c r="D46" t="n">
-        <v>10.12672943228455</v>
+        <v>84.17788762634217</v>
       </c>
       <c r="E46" t="n">
-        <v>60.35375930417172</v>
+        <v>31.98775817375721</v>
       </c>
       <c r="F46" t="n">
-        <v>16.02141069150186</v>
+        <v>46.81851215004129</v>
       </c>
       <c r="G46" t="n">
-        <v>178.0405379331909</v>
+        <v>179.0448983620993</v>
       </c>
       <c r="H46" t="n">
-        <v>155.9771685261542</v>
+        <v>176.4935139559854</v>
       </c>
     </row>
     <row r="47">
@@ -1626,25 +1626,25 @@
         <v>45</v>
       </c>
       <c r="B47" t="n">
-        <v>1.904994</v>
+        <v>3.706125</v>
       </c>
       <c r="C47" t="n">
-        <v>19.89008403944117</v>
+        <v>53.26656348902645</v>
       </c>
       <c r="D47" t="n">
-        <v>9.375693278328935</v>
+        <v>83.96795858715025</v>
       </c>
       <c r="E47" t="n">
-        <v>25.49238273872072</v>
+        <v>32.47149357769957</v>
       </c>
       <c r="F47" t="n">
-        <v>14.09053428992233</v>
+        <v>47.52687780704323</v>
       </c>
       <c r="G47" t="n">
-        <v>178.9277711214402</v>
+        <v>178.2554824172695</v>
       </c>
       <c r="H47" t="n">
-        <v>178.7639203661078</v>
+        <v>175.2675123410712</v>
       </c>
     </row>
     <row r="48">
@@ -1652,25 +1652,25 @@
         <v>46</v>
       </c>
       <c r="B48" t="n">
-        <v>1.939332</v>
+        <v>3.7759</v>
       </c>
       <c r="C48" t="n">
-        <v>18.6363008997886</v>
+        <v>53.6232060908082</v>
       </c>
       <c r="D48" t="n">
-        <v>9.823502468980273</v>
+        <v>83.74482161459898</v>
       </c>
       <c r="E48" t="n">
-        <v>43.25045387677648</v>
+        <v>32.7951960475982</v>
       </c>
       <c r="F48" t="n">
-        <v>13.52376995594678</v>
+        <v>47.47309033103875</v>
       </c>
       <c r="G48" t="n">
-        <v>177.9591759140422</v>
+        <v>177.6092896174584</v>
       </c>
       <c r="H48" t="n">
-        <v>168.9813688897079</v>
+        <v>174.821873502045</v>
       </c>
     </row>
     <row r="49">
@@ -1678,25 +1678,25 @@
         <v>47</v>
       </c>
       <c r="B49" t="n">
-        <v>1.973957</v>
+        <v>3.844815</v>
       </c>
       <c r="C49" t="n">
-        <v>23.78436081540821</v>
+        <v>66.09412023483289</v>
       </c>
       <c r="D49" t="n">
-        <v>11.82582610705993</v>
+        <v>81.9443470782025</v>
       </c>
       <c r="E49" t="n">
-        <v>27.34574469686651</v>
+        <v>47.7201267871126</v>
       </c>
       <c r="F49" t="n">
-        <v>16.33939306399088</v>
+        <v>48.45233667592522</v>
       </c>
       <c r="G49" t="n">
-        <v>177.8470627383124</v>
+        <v>175.3184166918535</v>
       </c>
       <c r="H49" t="n">
-        <v>179.4443273697571</v>
+        <v>164.9595265662568</v>
       </c>
     </row>
     <row r="50">
@@ -1704,25 +1704,25 @@
         <v>48</v>
       </c>
       <c r="B50" t="n">
-        <v>2.007086</v>
+        <v>3.915876</v>
       </c>
       <c r="C50" t="n">
-        <v>31.15652551922632</v>
+        <v>62.75668436516524</v>
       </c>
       <c r="D50" t="n">
-        <v>12.99597023579003</v>
+        <v>80.32532586403099</v>
       </c>
       <c r="E50" t="n">
-        <v>31.53078478009891</v>
+        <v>46.52824930439956</v>
       </c>
       <c r="F50" t="n">
-        <v>15.82260778604303</v>
+        <v>51.77033105500215</v>
       </c>
       <c r="G50" t="n">
-        <v>179.1568348504395</v>
+        <v>172.1647669094138</v>
       </c>
       <c r="H50" t="n">
-        <v>177.3364704812714</v>
+        <v>174.61749359083</v>
       </c>
     </row>
     <row r="51">
@@ -1730,25 +1730,25 @@
         <v>49</v>
       </c>
       <c r="B51" t="n">
-        <v>2.040343</v>
+        <v>3.985182</v>
       </c>
       <c r="C51" t="n">
-        <v>32.29018647470784</v>
+        <v>61.16900521526241</v>
       </c>
       <c r="D51" t="n">
-        <v>12.14966512240465</v>
+        <v>79.60449404648202</v>
       </c>
       <c r="E51" t="n">
-        <v>28.0942903454398</v>
+        <v>46.18827234914753</v>
       </c>
       <c r="F51" t="n">
-        <v>16.50433949812901</v>
+        <v>52.53574429422143</v>
       </c>
       <c r="G51" t="n">
-        <v>178.3092420867724</v>
+        <v>172.0621536256548</v>
       </c>
       <c r="H51" t="n">
-        <v>177.8091738897889</v>
+        <v>174.3877342589367</v>
       </c>
     </row>
     <row r="52">
@@ -1756,25 +1756,25 @@
         <v>50</v>
       </c>
       <c r="B52" t="n">
-        <v>2.073569</v>
+        <v>4.054312</v>
       </c>
       <c r="C52" t="n">
-        <v>35.19498716927824</v>
+        <v>62.76760933102233</v>
       </c>
       <c r="D52" t="n">
-        <v>13.02689103205894</v>
+        <v>77.97235674206804</v>
       </c>
       <c r="E52" t="n">
-        <v>35.6811867628911</v>
+        <v>50.13642099863272</v>
       </c>
       <c r="F52" t="n">
-        <v>17.83685092633485</v>
+        <v>57.41463140351099</v>
       </c>
       <c r="G52" t="n">
-        <v>178.7393506348704</v>
+        <v>171.9160920033247</v>
       </c>
       <c r="H52" t="n">
-        <v>168.2488070006076</v>
+        <v>168.4231771618758</v>
       </c>
     </row>
     <row r="53">
@@ -1782,25 +1782,25 @@
         <v>51</v>
       </c>
       <c r="B53" t="n">
-        <v>2.108276</v>
+        <v>4.122397</v>
       </c>
       <c r="C53" t="n">
-        <v>33.894428839358</v>
+        <v>34.55990465552091</v>
       </c>
       <c r="D53" t="n">
-        <v>13.91890849379924</v>
+        <v>77.7389488549972</v>
       </c>
       <c r="E53" t="n">
-        <v>34.81024983045137</v>
+        <v>147.6763379341931</v>
       </c>
       <c r="F53" t="n">
-        <v>20.12402374932693</v>
+        <v>60.21759959970549</v>
       </c>
       <c r="G53" t="n">
-        <v>179.0278968343008</v>
+        <v>173.6072241823734</v>
       </c>
       <c r="H53" t="n">
-        <v>171.8823717084586</v>
+        <v>169.1511948335465</v>
       </c>
     </row>
     <row r="54">
@@ -1808,25 +1808,25 @@
         <v>52</v>
       </c>
       <c r="B54" t="n">
-        <v>2.146358</v>
+        <v>4.195778</v>
       </c>
       <c r="C54" t="n">
-        <v>36.05881443421627</v>
+        <v>52.17063033203627</v>
       </c>
       <c r="D54" t="n">
-        <v>13.99283460641204</v>
+        <v>77.5429981842742</v>
       </c>
       <c r="E54" t="n">
-        <v>32.82603758365597</v>
+        <v>43.52873788203408</v>
       </c>
       <c r="F54" t="n">
-        <v>21.06890741133921</v>
+        <v>60.43750420778888</v>
       </c>
       <c r="G54" t="n">
-        <v>179.2153197893783</v>
+        <v>172.1930482570437</v>
       </c>
       <c r="H54" t="n">
-        <v>160.1793728857634</v>
+        <v>175.2878305614128</v>
       </c>
     </row>
     <row r="55">
@@ -1834,25 +1834,25 @@
         <v>53</v>
       </c>
       <c r="B55" t="n">
-        <v>2.181191</v>
+        <v>4.266</v>
       </c>
       <c r="C55" t="n">
-        <v>36.5932758367252</v>
+        <v>52.73559014390679</v>
       </c>
       <c r="D55" t="n">
-        <v>14.81007827372418</v>
+        <v>77.31793215688116</v>
       </c>
       <c r="E55" t="n">
-        <v>29.61228066539555</v>
+        <v>54.57594585975186</v>
       </c>
       <c r="F55" t="n">
-        <v>20.68083999543693</v>
+        <v>60.68170094237417</v>
       </c>
       <c r="G55" t="n">
-        <v>178.8503720666277</v>
+        <v>172.7194932225054</v>
       </c>
       <c r="H55" t="n">
-        <v>170.5107207807561</v>
+        <v>165.1430058335851</v>
       </c>
     </row>
     <row r="56">
@@ -1860,25 +1860,25 @@
         <v>54</v>
       </c>
       <c r="B56" t="n">
-        <v>2.216599</v>
+        <v>4.339287</v>
       </c>
       <c r="C56" t="n">
-        <v>32.39378830445649</v>
+        <v>62.5268815838252</v>
       </c>
       <c r="D56" t="n">
-        <v>14.84452989667108</v>
+        <v>76.81740661143185</v>
       </c>
       <c r="E56" t="n">
-        <v>31.78735357864429</v>
+        <v>56.0887380333433</v>
       </c>
       <c r="F56" t="n">
-        <v>15.81690211939819</v>
+        <v>59.53535598293234</v>
       </c>
       <c r="G56" t="n">
-        <v>174.5018712190842</v>
+        <v>172.4448352588007</v>
       </c>
       <c r="H56" t="n">
-        <v>165.4308317117359</v>
+        <v>168.8150696514589</v>
       </c>
     </row>
     <row r="57">
@@ -1886,25 +1886,25 @@
         <v>55</v>
       </c>
       <c r="B57" t="n">
-        <v>2.254211</v>
+        <v>4.407803</v>
       </c>
       <c r="C57" t="n">
-        <v>31.16254351301217</v>
+        <v>65.4422056537594</v>
       </c>
       <c r="D57" t="n">
-        <v>14.64942360601711</v>
+        <v>75.52659256009295</v>
       </c>
       <c r="E57" t="n">
-        <v>42.15849164194764</v>
+        <v>54.17259512332456</v>
       </c>
       <c r="F57" t="n">
-        <v>24.24025529092409</v>
+        <v>57.31703757585498</v>
       </c>
       <c r="G57" t="n">
-        <v>165.722483236918</v>
+        <v>172.7419838806688</v>
       </c>
       <c r="H57" t="n">
-        <v>161.8457819047264</v>
+        <v>156.5991547307111</v>
       </c>
     </row>
     <row r="58">
@@ -1912,25 +1912,25 @@
         <v>56</v>
       </c>
       <c r="B58" t="n">
-        <v>2.288258</v>
+        <v>4.476565</v>
       </c>
       <c r="C58" t="n">
-        <v>26.2430631877698</v>
+        <v>67.17143054023636</v>
       </c>
       <c r="D58" t="n">
-        <v>13.54990163531656</v>
+        <v>74.54841140819318</v>
       </c>
       <c r="E58" t="n">
-        <v>140.6276589427137</v>
+        <v>53.42995297820107</v>
       </c>
       <c r="F58" t="n">
-        <v>137.9634484657681</v>
+        <v>55.97154904017535</v>
       </c>
       <c r="G58" t="n">
-        <v>153.3526154249068</v>
+        <v>173.3871778637944</v>
       </c>
       <c r="H58" t="n">
-        <v>118.1606719157625</v>
+        <v>154.8069055022883</v>
       </c>
     </row>
     <row r="59">
@@ -1938,25 +1938,25 @@
         <v>57</v>
       </c>
       <c r="B59" t="n">
-        <v>2.323634</v>
+        <v>4.556299</v>
       </c>
       <c r="C59" t="n">
-        <v>24.66019250223411</v>
+        <v>62.96278780258809</v>
       </c>
       <c r="D59" t="n">
-        <v>14.78716992563427</v>
+        <v>71.59797502204653</v>
       </c>
       <c r="E59" t="n">
-        <v>124.7356378572265</v>
+        <v>46.99115648655318</v>
       </c>
       <c r="F59" t="n">
-        <v>86.2537301881156</v>
+        <v>51.38524773419383</v>
       </c>
       <c r="G59" t="n">
-        <v>134.9257492087062</v>
+        <v>173.7937467260773</v>
       </c>
       <c r="H59" t="n">
-        <v>146.9025943401089</v>
+        <v>154.4231583099995</v>
       </c>
     </row>
     <row r="60">
@@ -1964,25 +1964,25 @@
         <v>58</v>
       </c>
       <c r="B60" t="n">
-        <v>2.37092</v>
+        <v>4.614963</v>
       </c>
       <c r="C60" t="n">
-        <v>24.72781018056937</v>
+        <v>54.74178086846883</v>
       </c>
       <c r="D60" t="n">
-        <v>14.320921004217</v>
+        <v>69.00755174941817</v>
       </c>
       <c r="E60" t="n">
-        <v>138.2262250212986</v>
+        <v>37.43442097047014</v>
       </c>
       <c r="F60" t="n">
-        <v>153.0131109572882</v>
+        <v>48.07343499247357</v>
       </c>
       <c r="G60" t="n">
-        <v>166.3787107214503</v>
+        <v>173.5945898319346</v>
       </c>
       <c r="H60" t="n">
-        <v>172.3158859883432</v>
+        <v>168.2549540783127</v>
       </c>
     </row>
     <row r="61">
@@ -1990,25 +1990,25 @@
         <v>59</v>
       </c>
       <c r="B61" t="n">
-        <v>2.404579</v>
+        <v>4.685754</v>
       </c>
       <c r="C61" t="n">
-        <v>25.17849583961461</v>
+        <v>51.97065439781998</v>
       </c>
       <c r="D61" t="n">
-        <v>14.48188077913054</v>
+        <v>67.99043092568824</v>
       </c>
       <c r="E61" t="n">
-        <v>129.3876128390564</v>
+        <v>34.23883654116269</v>
       </c>
       <c r="F61" t="n">
-        <v>136.5656748165545</v>
+        <v>46.57569955069224</v>
       </c>
       <c r="G61" t="n">
-        <v>153.7556265736854</v>
+        <v>173.0365683908047</v>
       </c>
       <c r="H61" t="n">
-        <v>158.7555726250465</v>
+        <v>173.0463559470954</v>
       </c>
     </row>
     <row r="62">
@@ -2016,25 +2016,25 @@
         <v>60</v>
       </c>
       <c r="B62" t="n">
-        <v>2.439232</v>
+        <v>4.740913</v>
       </c>
       <c r="C62" t="n">
-        <v>23.77068055852879</v>
+        <v>50.12373097315212</v>
       </c>
       <c r="D62" t="n">
-        <v>14.0434507658525</v>
+        <v>55.9568071584433</v>
       </c>
       <c r="E62" t="n">
-        <v>48.7728674061201</v>
+        <v>34.46937624271989</v>
       </c>
       <c r="F62" t="n">
-        <v>153.2642314111347</v>
+        <v>41.19835939175614</v>
       </c>
       <c r="G62" t="n">
-        <v>167.3272088947122</v>
+        <v>175.5106023711001</v>
       </c>
       <c r="H62" t="n">
-        <v>117.392473436587</v>
+        <v>168.9512466318485</v>
       </c>
     </row>
     <row r="63">
@@ -2042,25 +2042,25 @@
         <v>61</v>
       </c>
       <c r="B63" t="n">
-        <v>2.471936</v>
+        <v>4.812208</v>
       </c>
       <c r="C63" t="n">
-        <v>27.23794344807015</v>
+        <v>47.985397665641</v>
       </c>
       <c r="D63" t="n">
-        <v>14.35486334521976</v>
+        <v>49.13602818950135</v>
       </c>
       <c r="E63" t="n">
-        <v>12.04815577178535</v>
+        <v>35.46864520748069</v>
       </c>
       <c r="F63" t="n">
-        <v>139.0838252791162</v>
+        <v>47.75445361632499</v>
       </c>
       <c r="G63" t="n">
-        <v>144.5695794805614</v>
+        <v>174.5463138088177</v>
       </c>
       <c r="H63" t="n">
-        <v>174.9930931320573</v>
+        <v>165.6375178011918</v>
       </c>
     </row>
     <row r="64">
@@ -2068,25 +2068,25 @@
         <v>62</v>
       </c>
       <c r="B64" t="n">
-        <v>2.505505</v>
+        <v>4.865131</v>
       </c>
       <c r="C64" t="n">
-        <v>27.09583049474271</v>
+        <v>46.37149119961036</v>
       </c>
       <c r="D64" t="n">
-        <v>14.11185291190791</v>
+        <v>48.05473759684359</v>
       </c>
       <c r="E64" t="n">
-        <v>13.93102798459608</v>
+        <v>37.00351066273771</v>
       </c>
       <c r="F64" t="n">
-        <v>149.9179390278913</v>
+        <v>50.56578810627527</v>
       </c>
       <c r="G64" t="n">
-        <v>166.7275908178835</v>
+        <v>171.1395951466926</v>
       </c>
       <c r="H64" t="n">
-        <v>174.2503301059428</v>
+        <v>162.2558409754711</v>
       </c>
     </row>
     <row r="65">
@@ -2094,25 +2094,25 @@
         <v>63</v>
       </c>
       <c r="B65" t="n">
-        <v>2.540561</v>
+        <v>4.936892</v>
       </c>
       <c r="C65" t="n">
-        <v>26.85935471231677</v>
+        <v>49.10688164509492</v>
       </c>
       <c r="D65" t="n">
-        <v>14.63233570939297</v>
+        <v>36.80987030781105</v>
       </c>
       <c r="E65" t="n">
-        <v>15.13278032082725</v>
+        <v>40.12273733392811</v>
       </c>
       <c r="F65" t="n">
-        <v>145.9219177041961</v>
+        <v>78.85505008389286</v>
       </c>
       <c r="G65" t="n">
-        <v>157.8186456356865</v>
+        <v>149.3808576878694</v>
       </c>
       <c r="H65" t="n">
-        <v>171.3138009490407</v>
+        <v>169.2684646195817</v>
       </c>
     </row>
     <row r="66">
@@ -2120,25 +2120,25 @@
         <v>64</v>
       </c>
       <c r="B66" t="n">
-        <v>2.575155</v>
+        <v>5.007956</v>
       </c>
       <c r="C66" t="n">
-        <v>27.768011428612</v>
+        <v>32.62023751431035</v>
       </c>
       <c r="D66" t="n">
-        <v>15.14717593066764</v>
+        <v>29.38226943637645</v>
       </c>
       <c r="E66" t="n">
-        <v>13.45033991072314</v>
+        <v>147.0825708643829</v>
       </c>
       <c r="F66" t="n">
-        <v>145.1039199096688</v>
+        <v>100.15789891802</v>
       </c>
       <c r="G66" t="n">
-        <v>122.1071311606712</v>
+        <v>137.1602387708887</v>
       </c>
       <c r="H66" t="n">
-        <v>173.3019220028393</v>
+        <v>151.4402027089267</v>
       </c>
     </row>
     <row r="67">
@@ -2146,25 +2146,25 @@
         <v>65</v>
       </c>
       <c r="B67" t="n">
-        <v>2.612191</v>
+        <v>5.08973</v>
       </c>
       <c r="C67" t="n">
-        <v>32.02690816414516</v>
+        <v>28.87806612368331</v>
       </c>
       <c r="D67" t="n">
-        <v>15.03019583384841</v>
+        <v>28.41294418388909</v>
       </c>
       <c r="E67" t="n">
-        <v>13.35331405005086</v>
+        <v>152.5271535110618</v>
       </c>
       <c r="F67" t="n">
-        <v>142.7125011368075</v>
+        <v>103.2740415717602</v>
       </c>
       <c r="G67" t="n">
-        <v>122.4455322531157</v>
+        <v>136.6935537866508</v>
       </c>
       <c r="H67" t="n">
-        <v>172.6656646399866</v>
+        <v>157.7885280113798</v>
       </c>
     </row>
     <row r="68">
@@ -2172,25 +2172,25 @@
         <v>66</v>
       </c>
       <c r="B68" t="n">
-        <v>2.648266</v>
+        <v>5.147982</v>
       </c>
       <c r="C68" t="n">
-        <v>31.11760288196557</v>
+        <v>27.23173814460846</v>
       </c>
       <c r="D68" t="n">
-        <v>14.92509906941969</v>
+        <v>27.96170895329124</v>
       </c>
       <c r="E68" t="n">
-        <v>1.841295759685479</v>
+        <v>154.5398408130004</v>
       </c>
       <c r="F68" t="n">
-        <v>144.3904086005757</v>
+        <v>163.7828492842581</v>
       </c>
       <c r="G68" t="n">
-        <v>154.7560138633519</v>
+        <v>177.4269838028135</v>
       </c>
       <c r="H68" t="n">
-        <v>162.1420296925163</v>
+        <v>159.4101264564702</v>
       </c>
     </row>
     <row r="69">
@@ -2198,25 +2198,25 @@
         <v>67</v>
       </c>
       <c r="B69" t="n">
-        <v>2.683213</v>
+        <v>5.216133</v>
       </c>
       <c r="C69" t="n">
-        <v>30.85594879554187</v>
+        <v>27.34822936049065</v>
       </c>
       <c r="D69" t="n">
-        <v>14.82065248934519</v>
+        <v>24.54891969648882</v>
       </c>
       <c r="E69" t="n">
-        <v>2.241636770391455</v>
+        <v>156.0774421114095</v>
       </c>
       <c r="F69" t="n">
-        <v>132.731276431391</v>
+        <v>179.7599369495142</v>
       </c>
       <c r="G69" t="n">
-        <v>133.9219987777747</v>
+        <v>168.9151639138629</v>
       </c>
       <c r="H69" t="n">
-        <v>163.3157156496892</v>
+        <v>163.7938592564218</v>
       </c>
     </row>
     <row r="70">
@@ -2224,25 +2224,25 @@
         <v>68</v>
       </c>
       <c r="B70" t="n">
-        <v>2.716647</v>
+        <v>5.285999</v>
       </c>
       <c r="C70" t="n">
-        <v>27.89439271674142</v>
+        <v>30.4465238703105</v>
       </c>
       <c r="D70" t="n">
-        <v>14.55880911792797</v>
+        <v>24.31810010921439</v>
       </c>
       <c r="E70" t="n">
-        <v>2.946551034669822</v>
+        <v>160.2030555178924</v>
       </c>
       <c r="F70" t="n">
-        <v>128.7513354480349</v>
+        <v>177.5522536077612</v>
       </c>
       <c r="G70" t="n">
-        <v>139.9792255226612</v>
+        <v>168.6433109402443</v>
       </c>
       <c r="H70" t="n">
-        <v>165.6896923769004</v>
+        <v>159.5940481129443</v>
       </c>
     </row>
     <row r="71">
@@ -2250,25 +2250,25 @@
         <v>69</v>
       </c>
       <c r="B71" t="n">
-        <v>2.751411</v>
+        <v>5.356075</v>
       </c>
       <c r="C71" t="n">
-        <v>31.06930958382346</v>
+        <v>51.45083010219654</v>
       </c>
       <c r="D71" t="n">
-        <v>14.59568862839835</v>
+        <v>22.87526614881705</v>
       </c>
       <c r="E71" t="n">
-        <v>4.513554843966629</v>
+        <v>40.04469741874314</v>
       </c>
       <c r="F71" t="n">
-        <v>126.8365580133338</v>
+        <v>170.3898723868929</v>
       </c>
       <c r="G71" t="n">
-        <v>144.4342367770777</v>
+        <v>178.3854973053348</v>
       </c>
       <c r="H71" t="n">
-        <v>176.9631474297263</v>
+        <v>174.5834488461031</v>
       </c>
     </row>
     <row r="72">
@@ -2276,25 +2276,25 @@
         <v>70</v>
       </c>
       <c r="B72" t="n">
-        <v>2.784603</v>
+        <v>5.425197</v>
       </c>
       <c r="C72" t="n">
-        <v>45.75632036209747</v>
+        <v>49.64957755929957</v>
       </c>
       <c r="D72" t="n">
-        <v>16.24221496909054</v>
+        <v>21.20135631233299</v>
       </c>
       <c r="E72" t="n">
-        <v>7.915057228887816</v>
+        <v>43.99376283825141</v>
       </c>
       <c r="F72" t="n">
-        <v>31.59545603141642</v>
+        <v>167.0151817788529</v>
       </c>
       <c r="G72" t="n">
-        <v>175.7184694686001</v>
+        <v>178.4781882997052</v>
       </c>
       <c r="H72" t="n">
-        <v>157.0373944296115</v>
+        <v>157.0158958527273</v>
       </c>
     </row>
     <row r="73">
@@ -2302,25 +2302,25 @@
         <v>71</v>
       </c>
       <c r="B73" t="n">
-        <v>2.817638</v>
+        <v>5.499892</v>
       </c>
       <c r="C73" t="n">
-        <v>39.35062865037053</v>
+        <v>49.66172948911872</v>
       </c>
       <c r="D73" t="n">
-        <v>15.06691116187477</v>
+        <v>20.38986960707782</v>
       </c>
       <c r="E73" t="n">
-        <v>100.0007399853665</v>
+        <v>46.27332945056359</v>
       </c>
       <c r="F73" t="n">
-        <v>142.9739666759243</v>
+        <v>166.9178768616803</v>
       </c>
       <c r="G73" t="n">
-        <v>162.5057501826811</v>
+        <v>177.521795028252</v>
       </c>
       <c r="H73" t="n">
-        <v>132.8395889259218</v>
+        <v>156.6951876922895</v>
       </c>
     </row>
     <row r="74">
@@ -2328,25 +2328,25 @@
         <v>72</v>
       </c>
       <c r="B74" t="n">
-        <v>2.851126</v>
+        <v>5.563655</v>
       </c>
       <c r="C74" t="n">
-        <v>17.59203625229785</v>
+        <v>48.65896228092586</v>
       </c>
       <c r="D74" t="n">
-        <v>14.24875325239552</v>
+        <v>19.73450308412349</v>
       </c>
       <c r="E74" t="n">
-        <v>137.8909458291851</v>
+        <v>38.70422882689488</v>
       </c>
       <c r="F74" t="n">
-        <v>146.816189361146</v>
+        <v>168.451199897834</v>
       </c>
       <c r="G74" t="n">
-        <v>158.562140597164</v>
+        <v>178.9233842999373</v>
       </c>
       <c r="H74" t="n">
-        <v>155.7602010695838</v>
+        <v>166.2134484975053</v>
       </c>
     </row>
     <row r="75">
@@ -2354,25 +2354,25 @@
         <v>73</v>
       </c>
       <c r="B75" t="n">
-        <v>2.883832</v>
+        <v>5.632965</v>
       </c>
       <c r="C75" t="n">
-        <v>15.11200420623084</v>
+        <v>45.13791413156048</v>
       </c>
       <c r="D75" t="n">
-        <v>13.49856666933388</v>
+        <v>20.28401812420157</v>
       </c>
       <c r="E75" t="n">
-        <v>151.4387793232335</v>
+        <v>26.90752544184954</v>
       </c>
       <c r="F75" t="n">
-        <v>153.0302491772292</v>
+        <v>168.6926947130831</v>
       </c>
       <c r="G75" t="n">
-        <v>168.1238228935165</v>
+        <v>179.043509629636</v>
       </c>
       <c r="H75" t="n">
-        <v>170.9736457126289</v>
+        <v>174.7167466564326</v>
       </c>
     </row>
     <row r="76">
@@ -2380,25 +2380,25 @@
         <v>74</v>
       </c>
       <c r="B76" t="n">
-        <v>2.918458</v>
+        <v>5.702933</v>
       </c>
       <c r="C76" t="n">
-        <v>14.74233182852157</v>
+        <v>42.65683716403064</v>
       </c>
       <c r="D76" t="n">
-        <v>12.87516512186673</v>
+        <v>20.13043709565867</v>
       </c>
       <c r="E76" t="n">
-        <v>153.7651131956355</v>
+        <v>24.0917468592846</v>
       </c>
       <c r="F76" t="n">
-        <v>153.7313663450941</v>
+        <v>170.5070557824061</v>
       </c>
       <c r="G76" t="n">
-        <v>168.1171781425142</v>
+        <v>177.9862215406116</v>
       </c>
       <c r="H76" t="n">
-        <v>171.0855676723563</v>
+        <v>173.6562165997063</v>
       </c>
     </row>
     <row r="77">
@@ -2406,25 +2406,25 @@
         <v>75</v>
       </c>
       <c r="B77" t="n">
-        <v>2.952749</v>
+        <v>5.772977</v>
       </c>
       <c r="C77" t="n">
-        <v>14.75669175299798</v>
+        <v>39.75637829777323</v>
       </c>
       <c r="D77" t="n">
-        <v>12.51768506424549</v>
+        <v>18.72360982481348</v>
       </c>
       <c r="E77" t="n">
-        <v>153.46942705515</v>
+        <v>18.98487106139182</v>
       </c>
       <c r="F77" t="n">
-        <v>154.8017237420182</v>
+        <v>168.7214093360764</v>
       </c>
       <c r="G77" t="n">
-        <v>167.5813823796809</v>
+        <v>178.6280794138364</v>
       </c>
       <c r="H77" t="n">
-        <v>170.1220084380539</v>
+        <v>177.5355496776542</v>
       </c>
     </row>
     <row r="78">
@@ -2432,25 +2432,25 @@
         <v>76</v>
       </c>
       <c r="B78" t="n">
-        <v>2.986979</v>
+        <v>5.842399</v>
       </c>
       <c r="C78" t="n">
-        <v>15.0608076873225</v>
+        <v>43.49850079212984</v>
       </c>
       <c r="D78" t="n">
-        <v>11.97728609711419</v>
+        <v>17.46823035297187</v>
       </c>
       <c r="E78" t="n">
-        <v>149.0249295731141</v>
+        <v>18.50926252534352</v>
       </c>
       <c r="F78" t="n">
-        <v>152.1775250517891</v>
+        <v>168.5643611083554</v>
       </c>
       <c r="G78" t="n">
-        <v>164.3027379084922</v>
+        <v>176.9443873968181</v>
       </c>
       <c r="H78" t="n">
-        <v>164.9831827540721</v>
+        <v>179.4769896061108</v>
       </c>
     </row>
     <row r="79">
@@ -2458,25 +2458,25 @@
         <v>77</v>
       </c>
       <c r="B79" t="n">
-        <v>3.028132</v>
+        <v>5.916178</v>
       </c>
       <c r="C79" t="n">
-        <v>13.76593899178271</v>
+        <v>41.31367839784234</v>
       </c>
       <c r="D79" t="n">
-        <v>11.78819095956682</v>
+        <v>17.109751778696</v>
       </c>
       <c r="E79" t="n">
-        <v>154.7190546251268</v>
+        <v>17.35968868595371</v>
       </c>
       <c r="F79" t="n">
-        <v>155.3205761176027</v>
+        <v>170.0518546161821</v>
       </c>
       <c r="G79" t="n">
-        <v>171.0875485641151</v>
+        <v>177.1607011900603</v>
       </c>
       <c r="H79" t="n">
-        <v>171.5452680898835</v>
+        <v>179.5150921977181</v>
       </c>
     </row>
     <row r="80">
@@ -2484,25 +2484,25 @@
         <v>78</v>
       </c>
       <c r="B80" t="n">
-        <v>3.062696</v>
+        <v>5.998253</v>
       </c>
       <c r="C80" t="n">
-        <v>13.16032317967915</v>
+        <v>41.63034265832831</v>
       </c>
       <c r="D80" t="n">
-        <v>11.61273232385647</v>
+        <v>16.25334295616831</v>
       </c>
       <c r="E80" t="n">
-        <v>155.8903842287203</v>
+        <v>16.78358618592541</v>
       </c>
       <c r="F80" t="n">
-        <v>156.3489832108622</v>
+        <v>170.74095973773</v>
       </c>
       <c r="G80" t="n">
-        <v>171.3241612736302</v>
+        <v>178.006772448047</v>
       </c>
       <c r="H80" t="n">
-        <v>171.2114161655614</v>
+        <v>177.8489011716277</v>
       </c>
     </row>
     <row r="81">
@@ -2510,25 +2510,25 @@
         <v>79</v>
       </c>
       <c r="B81" t="n">
-        <v>3.095925</v>
+        <v>6.076771</v>
       </c>
       <c r="C81" t="n">
-        <v>12.80079193009566</v>
+        <v>44.1542533676454</v>
       </c>
       <c r="D81" t="n">
-        <v>11.54729379266789</v>
+        <v>15.36440469632419</v>
       </c>
       <c r="E81" t="n">
-        <v>156.2559749927648</v>
+        <v>21.8536955251965</v>
       </c>
       <c r="F81" t="n">
-        <v>157.967710210287</v>
+        <v>174.6236541118791</v>
       </c>
       <c r="G81" t="n">
-        <v>171.7057221057676</v>
+        <v>179.9249408092172</v>
       </c>
       <c r="H81" t="n">
-        <v>171.2879054275616</v>
+        <v>178.6143428183818</v>
       </c>
     </row>
     <row r="82">
@@ -2536,25 +2536,25 @@
         <v>80</v>
       </c>
       <c r="B82" t="n">
-        <v>3.130273</v>
+        <v>6.155642</v>
       </c>
       <c r="C82" t="n">
-        <v>12.72398106253259</v>
+        <v>47.34645991286249</v>
       </c>
       <c r="D82" t="n">
-        <v>11.39785120357429</v>
+        <v>15.14632142801831</v>
       </c>
       <c r="E82" t="n">
-        <v>156.2068452875692</v>
+        <v>26.06134367412442</v>
       </c>
       <c r="F82" t="n">
-        <v>159.096497325759</v>
+        <v>175.5149594500976</v>
       </c>
       <c r="G82" t="n">
-        <v>171.0383605772232</v>
+        <v>179.6457254781486</v>
       </c>
       <c r="H82" t="n">
-        <v>170.9147869712859</v>
+        <v>177.4813576316244</v>
       </c>
     </row>
     <row r="83">
@@ -2562,25 +2562,25 @@
         <v>81</v>
       </c>
       <c r="B83" t="n">
-        <v>3.16487</v>
+        <v>6.227792</v>
       </c>
       <c r="C83" t="n">
-        <v>11.94317662550775</v>
+        <v>49.11029643974842</v>
       </c>
       <c r="D83" t="n">
-        <v>11.44825538300745</v>
+        <v>15.32322640215654</v>
       </c>
       <c r="E83" t="n">
-        <v>151.3783214303084</v>
+        <v>27.77075305282402</v>
       </c>
       <c r="F83" t="n">
-        <v>158.8291350207305</v>
+        <v>176.0725582776884</v>
       </c>
       <c r="G83" t="n">
-        <v>169.2342570830503</v>
+        <v>178.6982105049374</v>
       </c>
       <c r="H83" t="n">
-        <v>158.7664912767206</v>
+        <v>177.17439652401</v>
       </c>
     </row>
     <row r="84">
@@ -2588,25 +2588,25 @@
         <v>82</v>
       </c>
       <c r="B84" t="n">
-        <v>3.199508</v>
+        <v>6.302861</v>
       </c>
       <c r="C84" t="n">
-        <v>11.64001758867554</v>
+        <v>45.92921612545803</v>
       </c>
       <c r="D84" t="n">
-        <v>11.28677187902984</v>
+        <v>14.71959782767507</v>
       </c>
       <c r="E84" t="n">
-        <v>155.5929305179839</v>
+        <v>37.90531094947272</v>
       </c>
       <c r="F84" t="n">
-        <v>159.2825016116176</v>
+        <v>176.5273428045866</v>
       </c>
       <c r="G84" t="n">
-        <v>170.0733797241569</v>
+        <v>177.4187889135911</v>
       </c>
       <c r="H84" t="n">
-        <v>173.0949127514001</v>
+        <v>165.7063043314478</v>
       </c>
     </row>
     <row r="85">
@@ -2614,25 +2614,25 @@
         <v>83</v>
       </c>
       <c r="B85" t="n">
-        <v>3.234402</v>
+        <v>6.370785</v>
       </c>
       <c r="C85" t="n">
-        <v>11.99989472892633</v>
+        <v>50.55719254778794</v>
       </c>
       <c r="D85" t="n">
-        <v>11.01899818600348</v>
+        <v>14.78194726597576</v>
       </c>
       <c r="E85" t="n">
-        <v>155.5829120924892</v>
+        <v>42.54543218118567</v>
       </c>
       <c r="F85" t="n">
-        <v>160.0103718087574</v>
+        <v>176.5402066481725</v>
       </c>
       <c r="G85" t="n">
-        <v>170.2971810316614</v>
+        <v>176.7077998452195</v>
       </c>
       <c r="H85" t="n">
-        <v>172.4257249337857</v>
+        <v>161.4427378407087</v>
       </c>
     </row>
     <row r="86">
@@ -2640,25 +2640,25 @@
         <v>84</v>
       </c>
       <c r="B86" t="n">
-        <v>3.26928</v>
+        <v>6.446792</v>
       </c>
       <c r="C86" t="n">
-        <v>11.40775681674902</v>
+        <v>51.22859474050298</v>
       </c>
       <c r="D86" t="n">
-        <v>10.63147747093026</v>
+        <v>15.17667857282169</v>
       </c>
       <c r="E86" t="n">
-        <v>157.9329227487663</v>
+        <v>42.0776738205651</v>
       </c>
       <c r="F86" t="n">
-        <v>160.6338512563898</v>
+        <v>175.8520904005883</v>
       </c>
       <c r="G86" t="n">
-        <v>171.3551455928945</v>
+        <v>176.8183293058633</v>
       </c>
       <c r="H86" t="n">
-        <v>172.7457781238531</v>
+        <v>164.0409105519037</v>
       </c>
     </row>
     <row r="87">
@@ -2666,25 +2666,25 @@
         <v>85</v>
       </c>
       <c r="B87" t="n">
-        <v>3.303414</v>
+        <v>6.518516</v>
       </c>
       <c r="C87" t="n">
-        <v>11.0114256971612</v>
+        <v>56.10927158602271</v>
       </c>
       <c r="D87" t="n">
-        <v>11.18997075210036</v>
+        <v>15.45433321018373</v>
       </c>
       <c r="E87" t="n">
-        <v>158.7489348614461</v>
+        <v>40.29433469631136</v>
       </c>
       <c r="F87" t="n">
-        <v>159.2576291065396</v>
+        <v>175.550452238053</v>
       </c>
       <c r="G87" t="n">
-        <v>169.6492293427592</v>
+        <v>179.9610793001642</v>
       </c>
       <c r="H87" t="n">
-        <v>172.4523104216039</v>
+        <v>169.7495882102077</v>
       </c>
     </row>
     <row r="88">
@@ -2692,25 +2692,25 @@
         <v>86</v>
       </c>
       <c r="B88" t="n">
-        <v>3.340222</v>
+        <v>6.598315</v>
       </c>
       <c r="C88" t="n">
-        <v>11.20469004865179</v>
+        <v>50.6205949314971</v>
       </c>
       <c r="D88" t="n">
-        <v>11.05419852198652</v>
+        <v>15.7980888788601</v>
       </c>
       <c r="E88" t="n">
-        <v>159.1016494184351</v>
+        <v>43.56827647399943</v>
       </c>
       <c r="F88" t="n">
-        <v>158.2375120114013</v>
+        <v>172.2786970898583</v>
       </c>
       <c r="G88" t="n">
-        <v>167.9601537600848</v>
+        <v>179.0956243454042</v>
       </c>
       <c r="H88" t="n">
-        <v>173.3516162768494</v>
+        <v>158.7553853878355</v>
       </c>
     </row>
     <row r="89">
@@ -2718,25 +2718,25 @@
         <v>87</v>
       </c>
       <c r="B89" t="n">
-        <v>3.376975</v>
+        <v>6.670898</v>
       </c>
       <c r="C89" t="n">
-        <v>11.4109438269966</v>
+        <v>45.00960283986682</v>
       </c>
       <c r="D89" t="n">
-        <v>11.18847051955453</v>
+        <v>16.60776546132175</v>
       </c>
       <c r="E89" t="n">
-        <v>158.9464523277211</v>
+        <v>39.6949676911528</v>
       </c>
       <c r="F89" t="n">
-        <v>157.9464198443689</v>
+        <v>173.0181595603352</v>
       </c>
       <c r="G89" t="n">
-        <v>167.7702588984203</v>
+        <v>179.2724259197396</v>
       </c>
       <c r="H89" t="n">
-        <v>173.1041403595378</v>
+        <v>154.0542425988068</v>
       </c>
     </row>
     <row r="90">
@@ -2744,25 +2744,25 @@
         <v>88</v>
       </c>
       <c r="B90" t="n">
-        <v>3.510207</v>
+        <v>6.735905</v>
       </c>
       <c r="C90" t="n">
-        <v>11.37891469196999</v>
+        <v>43.19620301073247</v>
       </c>
       <c r="D90" t="n">
-        <v>10.81757997299224</v>
+        <v>16.9715284019847</v>
       </c>
       <c r="E90" t="n">
-        <v>159.0221894213784</v>
+        <v>38.68922264073938</v>
       </c>
       <c r="F90" t="n">
-        <v>157.9894862887249</v>
+        <v>172.4128870740396</v>
       </c>
       <c r="G90" t="n">
-        <v>167.5168141321579</v>
+        <v>178.8010278432104</v>
       </c>
       <c r="H90" t="n">
-        <v>172.7753070565049</v>
+        <v>153.2479586145884</v>
       </c>
     </row>
     <row r="91">
@@ -2770,25 +2770,25 @@
         <v>89</v>
       </c>
       <c r="B91" t="n">
-        <v>3.545954</v>
+        <v>6.796709</v>
       </c>
       <c r="C91" t="n">
-        <v>11.3098738033344</v>
+        <v>43.14480364983771</v>
       </c>
       <c r="D91" t="n">
-        <v>10.69770719804255</v>
+        <v>17.19259158516947</v>
       </c>
       <c r="E91" t="n">
-        <v>159.5938087872401</v>
+        <v>36.30726668354173</v>
       </c>
       <c r="F91" t="n">
-        <v>159.3200531660196</v>
+        <v>172.2488026116936</v>
       </c>
       <c r="G91" t="n">
-        <v>168.7785804662006</v>
+        <v>179.5450366239146</v>
       </c>
       <c r="H91" t="n">
-        <v>173.4586809289187</v>
+        <v>162.2539508954309</v>
       </c>
     </row>
     <row r="92">
@@ -2796,25 +2796,25 @@
         <v>90</v>
       </c>
       <c r="B92" t="n">
-        <v>3.58043</v>
+        <v>6.865106</v>
       </c>
       <c r="C92" t="n">
-        <v>11.30432817769961</v>
+        <v>41.61991076526521</v>
       </c>
       <c r="D92" t="n">
-        <v>10.65398913925238</v>
+        <v>17.38902960086768</v>
       </c>
       <c r="E92" t="n">
-        <v>159.6130727664362</v>
+        <v>34.01709123763457</v>
       </c>
       <c r="F92" t="n">
-        <v>158.8880190589306</v>
+        <v>171.7688550704576</v>
       </c>
       <c r="G92" t="n">
-        <v>169.1320539702091</v>
+        <v>179.1554944182652</v>
       </c>
       <c r="H92" t="n">
-        <v>172.6925915822952</v>
+        <v>163.8598457294412</v>
       </c>
     </row>
     <row r="93">
@@ -2822,25 +2822,25 @@
         <v>91</v>
       </c>
       <c r="B93" t="n">
-        <v>3.615409</v>
+        <v>6.934726</v>
       </c>
       <c r="C93" t="n">
-        <v>11.34271082874494</v>
+        <v>41.15804201668009</v>
       </c>
       <c r="D93" t="n">
-        <v>10.63641286524402</v>
+        <v>17.56587945267641</v>
       </c>
       <c r="E93" t="n">
-        <v>159.681649070423</v>
+        <v>32.8994253373445</v>
       </c>
       <c r="F93" t="n">
-        <v>160.246348304818</v>
+        <v>171.354905466729</v>
       </c>
       <c r="G93" t="n">
-        <v>169.0854125905364</v>
+        <v>178.8969048029907</v>
       </c>
       <c r="H93" t="n">
-        <v>173.1163469333564</v>
+        <v>164.7307655888853</v>
       </c>
     </row>
     <row r="94">
@@ -2848,25 +2848,25 @@
         <v>92</v>
       </c>
       <c r="B94" t="n">
-        <v>3.650663</v>
+        <v>7.006352</v>
       </c>
       <c r="C94" t="n">
-        <v>11.39444951361869</v>
+        <v>40.27794896671811</v>
       </c>
       <c r="D94" t="n">
-        <v>10.70090030887839</v>
+        <v>17.54904880610439</v>
       </c>
       <c r="E94" t="n">
-        <v>160.1598807236018</v>
+        <v>32.34057908629961</v>
       </c>
       <c r="F94" t="n">
-        <v>160.3497613698937</v>
+        <v>172.0297294431047</v>
       </c>
       <c r="G94" t="n">
-        <v>168.5368038647564</v>
+        <v>179.3018762291029</v>
       </c>
       <c r="H94" t="n">
-        <v>172.8801101299019</v>
+        <v>165.6610070818608</v>
       </c>
     </row>
     <row r="95">
@@ -2874,25 +2874,25 @@
         <v>93</v>
       </c>
       <c r="B95" t="n">
-        <v>3.685004</v>
+        <v>7.066639</v>
       </c>
       <c r="C95" t="n">
-        <v>11.13939681948363</v>
+        <v>37.29671174365028</v>
       </c>
       <c r="D95" t="n">
-        <v>10.52014681397152</v>
+        <v>17.47772913046425</v>
       </c>
       <c r="E95" t="n">
-        <v>157.9046600413737</v>
+        <v>26.2014222607476</v>
       </c>
       <c r="F95" t="n">
-        <v>156.8134971411473</v>
+        <v>171.8413479255491</v>
       </c>
       <c r="G95" t="n">
-        <v>168.1894028383181</v>
+        <v>179.1198269195474</v>
       </c>
       <c r="H95" t="n">
-        <v>169.4376254432202</v>
+        <v>170.4426928405134</v>
       </c>
     </row>
     <row r="96">
@@ -2900,25 +2900,25 @@
         <v>94</v>
       </c>
       <c r="B96" t="n">
-        <v>3.720461</v>
+        <v>7.139351</v>
       </c>
       <c r="C96" t="n">
-        <v>10.82967110945824</v>
+        <v>37.51497398378416</v>
       </c>
       <c r="D96" t="n">
-        <v>10.60102243863528</v>
+        <v>17.42624998557323</v>
       </c>
       <c r="E96" t="n">
-        <v>157.9935307766388</v>
+        <v>25.33204498082339</v>
       </c>
       <c r="F96" t="n">
-        <v>154.0878873341799</v>
+        <v>171.7623430948738</v>
       </c>
       <c r="G96" t="n">
-        <v>162.7665021841686</v>
+        <v>178.9423570382561</v>
       </c>
       <c r="H96" t="n">
-        <v>168.9560645136494</v>
+        <v>172.0449081607054</v>
       </c>
     </row>
     <row r="97">
@@ -2926,25 +2926,25 @@
         <v>95</v>
       </c>
       <c r="B97" t="n">
-        <v>3.754875</v>
+        <v>7.195811</v>
       </c>
       <c r="C97" t="n">
-        <v>10.83057405800252</v>
+        <v>35.61340462537149</v>
       </c>
       <c r="D97" t="n">
-        <v>10.56675108453191</v>
+        <v>17.46059790457213</v>
       </c>
       <c r="E97" t="n">
-        <v>158.5909736250827</v>
+        <v>26.29343736418568</v>
       </c>
       <c r="F97" t="n">
-        <v>154.9976486657168</v>
+        <v>171.1545882328448</v>
       </c>
       <c r="G97" t="n">
-        <v>166.5201343294916</v>
+        <v>179.251259970724</v>
       </c>
       <c r="H97" t="n">
-        <v>172.5333477486511</v>
+        <v>171.5712537105725</v>
       </c>
     </row>
     <row r="98">
@@ -2952,25 +2952,25 @@
         <v>96</v>
       </c>
       <c r="B98" t="n">
-        <v>3.78951</v>
+        <v>7.268574</v>
       </c>
       <c r="C98" t="n">
-        <v>10.73459483046091</v>
+        <v>26.88694333516381</v>
       </c>
       <c r="D98" t="n">
-        <v>10.60082686319618</v>
+        <v>17.25381921744372</v>
       </c>
       <c r="E98" t="n">
-        <v>159.0639560528359</v>
+        <v>19.65807297586748</v>
       </c>
       <c r="F98" t="n">
-        <v>154.7180666914271</v>
+        <v>171.3546555718752</v>
       </c>
       <c r="G98" t="n">
-        <v>165.8909018647677</v>
+        <v>175.023728433748</v>
       </c>
       <c r="H98" t="n">
-        <v>172.806433789177</v>
+        <v>175.8348207494205</v>
       </c>
     </row>
     <row r="99">
@@ -2978,25 +2978,25 @@
         <v>97</v>
       </c>
       <c r="B99" t="n">
-        <v>3.8233</v>
+        <v>7.327314</v>
       </c>
       <c r="C99" t="n">
-        <v>10.60618136741397</v>
+        <v>25.53472686234842</v>
       </c>
       <c r="D99" t="n">
-        <v>10.07633008448056</v>
+        <v>17.07684543207512</v>
       </c>
       <c r="E99" t="n">
-        <v>152.25310793061</v>
+        <v>18.75473800569831</v>
       </c>
       <c r="F99" t="n">
-        <v>152.5106488001239</v>
+        <v>171.6807892408054</v>
       </c>
       <c r="G99" t="n">
-        <v>160.1812945474957</v>
+        <v>173.1564815009613</v>
       </c>
       <c r="H99" t="n">
-        <v>163.8849314532713</v>
+        <v>176.7955907048664</v>
       </c>
     </row>
     <row r="100">
@@ -3004,25 +3004,25 @@
         <v>98</v>
       </c>
       <c r="B100" t="n">
-        <v>3.860416</v>
+        <v>7.397566</v>
       </c>
       <c r="C100" t="n">
-        <v>10.50448556908134</v>
+        <v>15.62556747704982</v>
       </c>
       <c r="D100" t="n">
-        <v>10.15338548658458</v>
+        <v>16.60657530303423</v>
       </c>
       <c r="E100" t="n">
-        <v>155.8988564527055</v>
+        <v>3.751608459200373</v>
       </c>
       <c r="F100" t="n">
-        <v>153.3996449364552</v>
+        <v>170.4102732933358</v>
       </c>
       <c r="G100" t="n">
-        <v>161.2218430270719</v>
+        <v>167.7707365644274</v>
       </c>
       <c r="H100" t="n">
-        <v>173.4967487501073</v>
+        <v>175.8247716666907</v>
       </c>
     </row>
     <row r="101">
@@ -3030,25 +3030,25 @@
         <v>99</v>
       </c>
       <c r="B101" t="n">
-        <v>3.895793</v>
+        <v>7.467336</v>
       </c>
       <c r="C101" t="n">
-        <v>11.26849212654968</v>
+        <v>14.27272209273131</v>
       </c>
       <c r="D101" t="n">
-        <v>10.16115952404191</v>
+        <v>16.15952329377873</v>
       </c>
       <c r="E101" t="n">
-        <v>151.2007987962061</v>
+        <v>152.5984397221125</v>
       </c>
       <c r="F101" t="n">
-        <v>152.3140923506807</v>
+        <v>170.8657942922686</v>
       </c>
       <c r="G101" t="n">
-        <v>160.6089207485554</v>
+        <v>165.7928232127864</v>
       </c>
       <c r="H101" t="n">
-        <v>168.4994039305821</v>
+        <v>171.631580075807</v>
       </c>
     </row>
     <row r="102">
@@ -3056,25 +3056,25 @@
         <v>100</v>
       </c>
       <c r="B102" t="n">
-        <v>3.929555</v>
+        <v>7.540309</v>
       </c>
       <c r="C102" t="n">
-        <v>11.25357184946967</v>
+        <v>13.96289806274765</v>
       </c>
       <c r="D102" t="n">
-        <v>9.94930874136613</v>
+        <v>16.01951685494399</v>
       </c>
       <c r="E102" t="n">
-        <v>150.6063758777082</v>
+        <v>153.9747927622519</v>
       </c>
       <c r="F102" t="n">
-        <v>152.4077354000532</v>
+        <v>171.533062348046</v>
       </c>
       <c r="G102" t="n">
-        <v>161.6574775170218</v>
+        <v>165.223030236299</v>
       </c>
       <c r="H102" t="n">
-        <v>169.2480601356104</v>
+        <v>168.1403065354465</v>
       </c>
     </row>
     <row r="103">
@@ -3082,25 +3082,25 @@
         <v>101</v>
       </c>
       <c r="B103" t="n">
-        <v>3.963654</v>
+        <v>7.606164</v>
       </c>
       <c r="C103" t="n">
-        <v>11.45079100733808</v>
+        <v>13.12408116126307</v>
       </c>
       <c r="D103" t="n">
-        <v>10.11572231029782</v>
+        <v>15.84854768204736</v>
       </c>
       <c r="E103" t="n">
-        <v>151.9936949713651</v>
+        <v>158.6134165715849</v>
       </c>
       <c r="F103" t="n">
-        <v>146.03543577503</v>
+        <v>171.7817353507813</v>
       </c>
       <c r="G103" t="n">
-        <v>150.7879353850923</v>
+        <v>165.967614177926</v>
       </c>
       <c r="H103" t="n">
-        <v>169.7443123190987</v>
+        <v>179.615492789573</v>
       </c>
     </row>
     <row r="104">
@@ -3108,25 +3108,25 @@
         <v>102</v>
       </c>
       <c r="B104" t="n">
-        <v>3.998385</v>
+        <v>7.671761</v>
       </c>
       <c r="C104" t="n">
-        <v>11.84420292187979</v>
+        <v>13.65185015830892</v>
       </c>
       <c r="D104" t="n">
-        <v>10.08560520479605</v>
+        <v>15.66674477895942</v>
       </c>
       <c r="E104" t="n">
-        <v>155.939959194976</v>
+        <v>159.1549394200832</v>
       </c>
       <c r="F104" t="n">
-        <v>147.7624433189176</v>
+        <v>171.8843724957613</v>
       </c>
       <c r="G104" t="n">
-        <v>158.0094490238001</v>
+        <v>168.8408508146108</v>
       </c>
       <c r="H104" t="n">
-        <v>174.1352369830888</v>
+        <v>178.9998562521969</v>
       </c>
     </row>
     <row r="105">
@@ -3134,25 +3134,25 @@
         <v>103</v>
       </c>
       <c r="B105" t="n">
-        <v>4.032678</v>
+        <v>7.740906</v>
       </c>
       <c r="C105" t="n">
-        <v>12.01548339356023</v>
+        <v>14.03645561402342</v>
       </c>
       <c r="D105" t="n">
-        <v>9.84748243241949</v>
+        <v>15.64395255920903</v>
       </c>
       <c r="E105" t="n">
-        <v>146.2656943873187</v>
+        <v>159.1712226001576</v>
       </c>
       <c r="F105" t="n">
-        <v>148.2158571431539</v>
+        <v>171.8643870056878</v>
       </c>
       <c r="G105" t="n">
-        <v>158.6875778132121</v>
+        <v>170.1251651297984</v>
       </c>
       <c r="H105" t="n">
-        <v>158.3578377913154</v>
+        <v>179.288793083283</v>
       </c>
     </row>
     <row r="106">
@@ -3160,25 +3160,25 @@
         <v>104</v>
       </c>
       <c r="B106" t="n">
-        <v>4.066306</v>
+        <v>7.800373</v>
       </c>
       <c r="C106" t="n">
-        <v>12.03727539121226</v>
+        <v>13.20170235780283</v>
       </c>
       <c r="D106" t="n">
-        <v>9.74195285181608</v>
+        <v>15.38912525107094</v>
       </c>
       <c r="E106" t="n">
-        <v>143.9487577433093</v>
+        <v>161.5303864003956</v>
       </c>
       <c r="F106" t="n">
-        <v>118.2338809918778</v>
+        <v>172.9348963710299</v>
       </c>
       <c r="G106" t="n">
-        <v>131.2627379380804</v>
+        <v>172.4502793064348</v>
       </c>
       <c r="H106" t="n">
-        <v>154.1009498117689</v>
+        <v>177.2695268772896</v>
       </c>
     </row>
     <row r="107">
@@ -3186,25 +3186,25 @@
         <v>105</v>
       </c>
       <c r="B107" t="n">
-        <v>4.10138</v>
+        <v>7.871494</v>
       </c>
       <c r="C107" t="n">
-        <v>11.84487018277086</v>
+        <v>13.50798822829515</v>
       </c>
       <c r="D107" t="n">
-        <v>9.739398996671252</v>
+        <v>15.20837910722393</v>
       </c>
       <c r="E107" t="n">
-        <v>145.624489807906</v>
+        <v>160.8836242957326</v>
       </c>
       <c r="F107" t="n">
-        <v>130.7715102802701</v>
+        <v>172.9800170404755</v>
       </c>
       <c r="G107" t="n">
-        <v>143.9774537137786</v>
+        <v>172.2088639500489</v>
       </c>
       <c r="H107" t="n">
-        <v>165.1818792656613</v>
+        <v>178.3376404191492</v>
       </c>
     </row>
     <row r="108">
@@ -3212,25 +3212,25 @@
         <v>106</v>
       </c>
       <c r="B108" t="n">
-        <v>4.136752</v>
+        <v>7.928839</v>
       </c>
       <c r="C108" t="n">
-        <v>12.02752130242178</v>
+        <v>13.70587018468784</v>
       </c>
       <c r="D108" t="n">
-        <v>9.546769513825875</v>
+        <v>15.11809158737998</v>
       </c>
       <c r="E108" t="n">
-        <v>147.5160958708329</v>
+        <v>160.5117291697995</v>
       </c>
       <c r="F108" t="n">
-        <v>130.905524587478</v>
+        <v>172.9767710708902</v>
       </c>
       <c r="G108" t="n">
-        <v>140.6524490112505</v>
+        <v>172.1381206754533</v>
       </c>
       <c r="H108" t="n">
-        <v>167.290448394932</v>
+        <v>178.7403429694099</v>
       </c>
     </row>
     <row r="109">
@@ -3238,25 +3238,25 @@
         <v>107</v>
       </c>
       <c r="B109" t="n">
-        <v>4.171444</v>
+        <v>7.990557</v>
       </c>
       <c r="C109" t="n">
-        <v>11.96038073161275</v>
+        <v>13.09513579825144</v>
       </c>
       <c r="D109" t="n">
-        <v>8.975308845723061</v>
+        <v>15.16751191958406</v>
       </c>
       <c r="E109" t="n">
-        <v>154.3872595859943</v>
+        <v>161.8866706516815</v>
       </c>
       <c r="F109" t="n">
-        <v>146.214281948585</v>
+        <v>173.0591276846526</v>
       </c>
       <c r="G109" t="n">
-        <v>164.5059165154228</v>
+        <v>171.9625943437063</v>
       </c>
       <c r="H109" t="n">
-        <v>175.8364389378496</v>
+        <v>178.1998419554525</v>
       </c>
     </row>
     <row r="110">
@@ -3264,25 +3264,25 @@
         <v>108</v>
       </c>
       <c r="B110" t="n">
-        <v>4.204398</v>
+        <v>8.054867</v>
       </c>
       <c r="C110" t="n">
-        <v>11.9262496605459</v>
+        <v>12.77177852720557</v>
       </c>
       <c r="D110" t="n">
-        <v>9.346868468992225</v>
+        <v>15.20577218929419</v>
       </c>
       <c r="E110" t="n">
-        <v>150.6026677365633</v>
+        <v>162.8311616977276</v>
       </c>
       <c r="F110" t="n">
-        <v>138.5637522527307</v>
+        <v>173.1130698453564</v>
       </c>
       <c r="G110" t="n">
-        <v>146.5185563850548</v>
+        <v>171.7634739943873</v>
       </c>
       <c r="H110" t="n">
-        <v>163.999861209326</v>
+        <v>177.4156536060632</v>
       </c>
     </row>
     <row r="111">
@@ -3290,25 +3290,25 @@
         <v>109</v>
       </c>
       <c r="B111" t="n">
-        <v>4.239157</v>
+        <v>8.119578000000001</v>
       </c>
       <c r="C111" t="n">
-        <v>12.33514615056096</v>
+        <v>11.548382118961</v>
       </c>
       <c r="D111" t="n">
-        <v>9.32685510697255</v>
+        <v>15.22618141530587</v>
       </c>
       <c r="E111" t="n">
-        <v>145.9985086055542</v>
+        <v>165.3859128017795</v>
       </c>
       <c r="F111" t="n">
-        <v>107.3320705161358</v>
+        <v>172.678008167563</v>
       </c>
       <c r="G111" t="n">
-        <v>125.4101469921871</v>
+        <v>173.0165699938626</v>
       </c>
       <c r="H111" t="n">
-        <v>152.2668361029355</v>
+        <v>175.1421074360325</v>
       </c>
     </row>
     <row r="112">
@@ -3316,25 +3316,25 @@
         <v>110</v>
       </c>
       <c r="B112" t="n">
-        <v>4.274003</v>
+        <v>8.181998999999999</v>
       </c>
       <c r="C112" t="n">
-        <v>12.41088629482656</v>
+        <v>10.9313850663422</v>
       </c>
       <c r="D112" t="n">
-        <v>9.346644603914886</v>
+        <v>15.30592193440056</v>
       </c>
       <c r="E112" t="n">
-        <v>150.0637590561653</v>
+        <v>166.8724046595913</v>
       </c>
       <c r="F112" t="n">
-        <v>140.105861232729</v>
+        <v>172.1304597999164</v>
       </c>
       <c r="G112" t="n">
-        <v>155.6522097273939</v>
+        <v>173.0904567377034</v>
       </c>
       <c r="H112" t="n">
-        <v>170.7617301995343</v>
+        <v>173.9997154199973</v>
       </c>
     </row>
     <row r="113">
@@ -3342,25 +3342,25 @@
         <v>111</v>
       </c>
       <c r="B113" t="n">
-        <v>4.309836</v>
+        <v>8.253814999999999</v>
       </c>
       <c r="C113" t="n">
-        <v>12.37937759632668</v>
+        <v>10.66865973137398</v>
       </c>
       <c r="D113" t="n">
-        <v>10.03151537868881</v>
+        <v>15.36688514577211</v>
       </c>
       <c r="E113" t="n">
-        <v>151.1650336415146</v>
+        <v>167.5679097293417</v>
       </c>
       <c r="F113" t="n">
-        <v>152.0788768686512</v>
+        <v>171.7810401095764</v>
       </c>
       <c r="G113" t="n">
-        <v>166.0650513516036</v>
+        <v>173.1477741145436</v>
       </c>
       <c r="H113" t="n">
-        <v>172.8574900561528</v>
+        <v>173.3205803867372</v>
       </c>
     </row>
     <row r="114">
@@ -3368,25 +3368,25 @@
         <v>112</v>
       </c>
       <c r="B114" t="n">
-        <v>4.345091</v>
+        <v>8.316207</v>
       </c>
       <c r="C114" t="n">
-        <v>12.56765514086148</v>
+        <v>10.82355842496969</v>
       </c>
       <c r="D114" t="n">
-        <v>9.992800748499086</v>
+        <v>15.61355268821328</v>
       </c>
       <c r="E114" t="n">
-        <v>154.7570811648336</v>
+        <v>167.4589840240071</v>
       </c>
       <c r="F114" t="n">
-        <v>156.678130630415</v>
+        <v>169.7499935096667</v>
       </c>
       <c r="G114" t="n">
-        <v>170.6042736838562</v>
+        <v>173.7029022460951</v>
       </c>
       <c r="H114" t="n">
-        <v>174.304746579353</v>
+        <v>173.4014905455482</v>
       </c>
     </row>
     <row r="115">
@@ -3394,25 +3394,25 @@
         <v>113</v>
       </c>
       <c r="B115" t="n">
-        <v>4.381294</v>
+        <v>8.378806000000001</v>
       </c>
       <c r="C115" t="n">
-        <v>12.54818478181263</v>
+        <v>11.41923886375057</v>
       </c>
       <c r="D115" t="n">
-        <v>9.971229329585835</v>
+        <v>16.27571249067031</v>
       </c>
       <c r="E115" t="n">
-        <v>152.373666140869</v>
+        <v>166.5755359718594</v>
       </c>
       <c r="F115" t="n">
-        <v>156.4299757428093</v>
+        <v>170.4521748934864</v>
       </c>
       <c r="G115" t="n">
-        <v>167.1092433685187</v>
+        <v>173.466936419092</v>
       </c>
       <c r="H115" t="n">
-        <v>168.4887599594406</v>
+        <v>173.2830616255745</v>
       </c>
     </row>
     <row r="116">
@@ -3420,25 +3420,25 @@
         <v>114</v>
       </c>
       <c r="B116" t="n">
-        <v>4.416862</v>
+        <v>8.454647</v>
       </c>
       <c r="C116" t="n">
-        <v>12.08256332950347</v>
+        <v>11.57797795094198</v>
       </c>
       <c r="D116" t="n">
-        <v>10.05897108922499</v>
+        <v>16.5009651789263</v>
       </c>
       <c r="E116" t="n">
-        <v>154.1050560704152</v>
+        <v>166.3785326623281</v>
       </c>
       <c r="F116" t="n">
-        <v>158.3998910645861</v>
+        <v>170.7993909290974</v>
       </c>
       <c r="G116" t="n">
-        <v>167.4474452012368</v>
+        <v>173.4110377166922</v>
       </c>
       <c r="H116" t="n">
-        <v>169.4699984651246</v>
+        <v>172.8568948036671</v>
       </c>
     </row>
     <row r="117">
@@ -3446,25 +3446,25 @@
         <v>115</v>
       </c>
       <c r="B117" t="n">
-        <v>4.451458</v>
+        <v>8.52858</v>
       </c>
       <c r="C117" t="n">
-        <v>12.17047440964647</v>
+        <v>11.62352653152464</v>
       </c>
       <c r="D117" t="n">
-        <v>10.33478850267895</v>
+        <v>16.20250949530424</v>
       </c>
       <c r="E117" t="n">
-        <v>151.9516142106458</v>
+        <v>166.0734209955806</v>
       </c>
       <c r="F117" t="n">
-        <v>158.5099038768095</v>
+        <v>171.293022368371</v>
       </c>
       <c r="G117" t="n">
-        <v>168.8645514525964</v>
+        <v>173.2028477007272</v>
       </c>
       <c r="H117" t="n">
-        <v>166.8909728201943</v>
+        <v>172.140661344098</v>
       </c>
     </row>
     <row r="118">
@@ -3472,25 +3472,25 @@
         <v>116</v>
       </c>
       <c r="B118" t="n">
-        <v>4.486782</v>
+        <v>8.594863999999999</v>
       </c>
       <c r="C118" t="n">
-        <v>12.21374796223734</v>
+        <v>11.72342318308257</v>
       </c>
       <c r="D118" t="n">
-        <v>10.98046623015823</v>
+        <v>16.06676797641147</v>
       </c>
       <c r="E118" t="n">
-        <v>154.9403088247482</v>
+        <v>165.887392031131</v>
       </c>
       <c r="F118" t="n">
-        <v>156.5835660181632</v>
+        <v>171.4337672522583</v>
       </c>
       <c r="G118" t="n">
-        <v>168.2280977087654</v>
+        <v>173.1409477478562</v>
       </c>
       <c r="H118" t="n">
-        <v>172.1015611474232</v>
+        <v>171.9632886015432</v>
       </c>
     </row>
     <row r="119">
@@ -3498,25 +3498,25 @@
         <v>117</v>
       </c>
       <c r="B119" t="n">
-        <v>4.522561</v>
+        <v>8.665022</v>
       </c>
       <c r="C119" t="n">
-        <v>12.54982141756787</v>
+        <v>11.92190722740991</v>
       </c>
       <c r="D119" t="n">
-        <v>10.8953283080667</v>
+        <v>16.08168654894148</v>
       </c>
       <c r="E119" t="n">
-        <v>155.6064336120291</v>
+        <v>165.6857489249929</v>
       </c>
       <c r="F119" t="n">
-        <v>157.4874674848355</v>
+        <v>171.3282785691732</v>
       </c>
       <c r="G119" t="n">
-        <v>169.7902735365769</v>
+        <v>173.3392956361888</v>
       </c>
       <c r="H119" t="n">
-        <v>173.0444539699529</v>
+        <v>171.8406226775788</v>
       </c>
     </row>
     <row r="120">
@@ -3524,25 +3524,25 @@
         <v>118</v>
       </c>
       <c r="B120" t="n">
-        <v>4.558156</v>
+        <v>8.745051999999999</v>
       </c>
       <c r="C120" t="n">
-        <v>12.45874861019195</v>
+        <v>12.01424815798223</v>
       </c>
       <c r="D120" t="n">
-        <v>10.93545691457049</v>
+        <v>16.10965461309721</v>
       </c>
       <c r="E120" t="n">
-        <v>157.0867070717977</v>
+        <v>165.6172626274515</v>
       </c>
       <c r="F120" t="n">
-        <v>158.9864193060956</v>
+        <v>171.1988206638612</v>
       </c>
       <c r="G120" t="n">
-        <v>170.7789948297733</v>
+        <v>173.4889361770549</v>
       </c>
       <c r="H120" t="n">
-        <v>173.7804439715686</v>
+        <v>171.691571079766</v>
       </c>
     </row>
     <row r="121">
@@ -3550,25 +3550,25 @@
         <v>119</v>
       </c>
       <c r="B121" t="n">
-        <v>4.594906</v>
+        <v>8.816554</v>
       </c>
       <c r="C121" t="n">
-        <v>12.93554073863765</v>
+        <v>11.79816263562992</v>
       </c>
       <c r="D121" t="n">
-        <v>10.86448756123683</v>
+        <v>16.17471898819323</v>
       </c>
       <c r="E121" t="n">
-        <v>157.0557857978421</v>
+        <v>165.6909241727649</v>
       </c>
       <c r="F121" t="n">
-        <v>159.2847481371715</v>
+        <v>171.276181761826</v>
       </c>
       <c r="G121" t="n">
-        <v>168.9779761338038</v>
+        <v>173.9474032344105</v>
       </c>
       <c r="H121" t="n">
-        <v>173.2155429215488</v>
+        <v>171.1570765642323</v>
       </c>
     </row>
     <row r="122">
@@ -3576,25 +3576,25 @@
         <v>120</v>
       </c>
       <c r="B122" t="n">
-        <v>4.630764</v>
+        <v>8.876314000000001</v>
       </c>
       <c r="C122" t="n">
-        <v>12.58480066483544</v>
+        <v>11.71003970306258</v>
       </c>
       <c r="D122" t="n">
-        <v>10.338895656258</v>
+        <v>16.20775864587006</v>
       </c>
       <c r="E122" t="n">
-        <v>156.2025158049487</v>
+        <v>165.8070722593766</v>
       </c>
       <c r="F122" t="n">
-        <v>156.6734512466259</v>
+        <v>171.8513613616355</v>
       </c>
       <c r="G122" t="n">
-        <v>168.2961010386703</v>
+        <v>174.6852507190338</v>
       </c>
       <c r="H122" t="n">
-        <v>170.5465781559314</v>
+        <v>171.3227857484059</v>
       </c>
     </row>
     <row r="123">
@@ -3602,25 +3602,571 @@
         <v>121</v>
       </c>
       <c r="B123" t="n">
-        <v>4.66346</v>
+        <v>8.948164999999999</v>
       </c>
       <c r="C123" t="n">
-        <v>13.58072274449069</v>
+        <v>11.73433479723068</v>
       </c>
       <c r="D123" t="n">
-        <v>10.42570969557843</v>
+        <v>16.23022359129252</v>
       </c>
       <c r="E123" t="n">
-        <v>154.670324434858</v>
+        <v>165.9813176055324</v>
       </c>
       <c r="F123" t="n">
-        <v>157.6520478677637</v>
+        <v>172.1549079973801</v>
       </c>
       <c r="G123" t="n">
-        <v>166.7026089743012</v>
+        <v>174.8909080167542</v>
       </c>
       <c r="H123" t="n">
-        <v>169.784509718982</v>
+        <v>170.1761754876706</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="1" t="n">
+        <v>122</v>
+      </c>
+      <c r="B124" t="n">
+        <v>9.017810000000001</v>
+      </c>
+      <c r="C124" t="n">
+        <v>11.82202589879989</v>
+      </c>
+      <c r="D124" t="n">
+        <v>16.33245008805465</v>
+      </c>
+      <c r="E124" t="n">
+        <v>165.6899000977916</v>
+      </c>
+      <c r="F124" t="n">
+        <v>172.1199972972107</v>
+      </c>
+      <c r="G124" t="n">
+        <v>174.5922188624692</v>
+      </c>
+      <c r="H124" t="n">
+        <v>169.7144880312664</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="1" t="n">
+        <v>123</v>
+      </c>
+      <c r="B125" t="n">
+        <v>9.098585999999999</v>
+      </c>
+      <c r="C125" t="n">
+        <v>11.97704542172744</v>
+      </c>
+      <c r="D125" t="n">
+        <v>16.081935531505</v>
+      </c>
+      <c r="E125" t="n">
+        <v>165.401611190654</v>
+      </c>
+      <c r="F125" t="n">
+        <v>171.7315613043484</v>
+      </c>
+      <c r="G125" t="n">
+        <v>174.2461296655483</v>
+      </c>
+      <c r="H125" t="n">
+        <v>169.9742152521916</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="1" t="n">
+        <v>124</v>
+      </c>
+      <c r="B126" t="n">
+        <v>9.166672</v>
+      </c>
+      <c r="C126" t="n">
+        <v>12.07248764703081</v>
+      </c>
+      <c r="D126" t="n">
+        <v>15.95425956638396</v>
+      </c>
+      <c r="E126" t="n">
+        <v>165.2375239593014</v>
+      </c>
+      <c r="F126" t="n">
+        <v>171.5200347001663</v>
+      </c>
+      <c r="G126" t="n">
+        <v>174.1435711922335</v>
+      </c>
+      <c r="H126" t="n">
+        <v>170.1164861711549</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="1" t="n">
+        <v>125</v>
+      </c>
+      <c r="B127" t="n">
+        <v>9.240126</v>
+      </c>
+      <c r="C127" t="n">
+        <v>12.14455091406247</v>
+      </c>
+      <c r="D127" t="n">
+        <v>15.92435571918829</v>
+      </c>
+      <c r="E127" t="n">
+        <v>165.000793333981</v>
+      </c>
+      <c r="F127" t="n">
+        <v>171.5817544420587</v>
+      </c>
+      <c r="G127" t="n">
+        <v>174.259653542761</v>
+      </c>
+      <c r="H127" t="n">
+        <v>169.8833882526631</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="1" t="n">
+        <v>126</v>
+      </c>
+      <c r="B128" t="n">
+        <v>9.307083</v>
+      </c>
+      <c r="C128" t="n">
+        <v>12.36112072746698</v>
+      </c>
+      <c r="D128" t="n">
+        <v>15.70959715215201</v>
+      </c>
+      <c r="E128" t="n">
+        <v>164.5143871086752</v>
+      </c>
+      <c r="F128" t="n">
+        <v>171.7483586212011</v>
+      </c>
+      <c r="G128" t="n">
+        <v>174.1103610418172</v>
+      </c>
+      <c r="H128" t="n">
+        <v>169.9960340428959</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="1" t="n">
+        <v>127</v>
+      </c>
+      <c r="B129" t="n">
+        <v>9.382664999999999</v>
+      </c>
+      <c r="C129" t="n">
+        <v>12.58430945847013</v>
+      </c>
+      <c r="D129" t="n">
+        <v>15.59866951498985</v>
+      </c>
+      <c r="E129" t="n">
+        <v>164.0141994210624</v>
+      </c>
+      <c r="F129" t="n">
+        <v>171.8501658418539</v>
+      </c>
+      <c r="G129" t="n">
+        <v>174.0346436497058</v>
+      </c>
+      <c r="H129" t="n">
+        <v>170.1977949705692</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="1" t="n">
+        <v>128</v>
+      </c>
+      <c r="B130" t="n">
+        <v>9.450062000000001</v>
+      </c>
+      <c r="C130" t="n">
+        <v>12.52714308080883</v>
+      </c>
+      <c r="D130" t="n">
+        <v>15.34189622492861</v>
+      </c>
+      <c r="E130" t="n">
+        <v>163.8335368414908</v>
+      </c>
+      <c r="F130" t="n">
+        <v>172.5641196557203</v>
+      </c>
+      <c r="G130" t="n">
+        <v>174.1441902800225</v>
+      </c>
+      <c r="H130" t="n">
+        <v>170.2568366075612</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="1" t="n">
+        <v>129</v>
+      </c>
+      <c r="B131" t="n">
+        <v>9.517199</v>
+      </c>
+      <c r="C131" t="n">
+        <v>12.37722247187419</v>
+      </c>
+      <c r="D131" t="n">
+        <v>15.34932865210904</v>
+      </c>
+      <c r="E131" t="n">
+        <v>163.9846196181857</v>
+      </c>
+      <c r="F131" t="n">
+        <v>172.1497009965375</v>
+      </c>
+      <c r="G131" t="n">
+        <v>174.2649960067599</v>
+      </c>
+      <c r="H131" t="n">
+        <v>170.2006932208558</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="1" t="n">
+        <v>130</v>
+      </c>
+      <c r="B132" t="n">
+        <v>9.590355000000001</v>
+      </c>
+      <c r="C132" t="n">
+        <v>12.52405761838957</v>
+      </c>
+      <c r="D132" t="n">
+        <v>15.39934882361596</v>
+      </c>
+      <c r="E132" t="n">
+        <v>163.4396255269764</v>
+      </c>
+      <c r="F132" t="n">
+        <v>171.7328266743245</v>
+      </c>
+      <c r="G132" t="n">
+        <v>173.9996326621895</v>
+      </c>
+      <c r="H132" t="n">
+        <v>170.2660884778473</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="1" t="n">
+        <v>131</v>
+      </c>
+      <c r="B133" t="n">
+        <v>9.662086</v>
+      </c>
+      <c r="C133" t="n">
+        <v>12.6242599994102</v>
+      </c>
+      <c r="D133" t="n">
+        <v>15.42857445094756</v>
+      </c>
+      <c r="E133" t="n">
+        <v>163.0917675831163</v>
+      </c>
+      <c r="F133" t="n">
+        <v>171.3915008800954</v>
+      </c>
+      <c r="G133" t="n">
+        <v>173.9127204302766</v>
+      </c>
+      <c r="H133" t="n">
+        <v>170.2634652342026</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="1" t="n">
+        <v>132</v>
+      </c>
+      <c r="B134" t="n">
+        <v>9.733891</v>
+      </c>
+      <c r="C134" t="n">
+        <v>12.48078102672052</v>
+      </c>
+      <c r="D134" t="n">
+        <v>15.14885501467713</v>
+      </c>
+      <c r="E134" t="n">
+        <v>163.3463048951688</v>
+      </c>
+      <c r="F134" t="n">
+        <v>170.2175465457431</v>
+      </c>
+      <c r="G134" t="n">
+        <v>175.0831924884596</v>
+      </c>
+      <c r="H134" t="n">
+        <v>170.2643506553799</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="1" t="n">
+        <v>133</v>
+      </c>
+      <c r="B135" t="n">
+        <v>9.806596000000001</v>
+      </c>
+      <c r="C135" t="n">
+        <v>12.31349758792129</v>
+      </c>
+      <c r="D135" t="n">
+        <v>15.00902586008274</v>
+      </c>
+      <c r="E135" t="n">
+        <v>163.791732642067</v>
+      </c>
+      <c r="F135" t="n">
+        <v>170.8549502021274</v>
+      </c>
+      <c r="G135" t="n">
+        <v>174.8499550425719</v>
+      </c>
+      <c r="H135" t="n">
+        <v>170.6207535408215</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="1" t="n">
+        <v>134</v>
+      </c>
+      <c r="B136" t="n">
+        <v>9.8752</v>
+      </c>
+      <c r="C136" t="n">
+        <v>12.194221945361</v>
+      </c>
+      <c r="D136" t="n">
+        <v>14.80279589662762</v>
+      </c>
+      <c r="E136" t="n">
+        <v>164.1149404268327</v>
+      </c>
+      <c r="F136" t="n">
+        <v>171.4543826733619</v>
+      </c>
+      <c r="G136" t="n">
+        <v>174.4859079521478</v>
+      </c>
+      <c r="H136" t="n">
+        <v>170.829392219705</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="1" t="n">
+        <v>135</v>
+      </c>
+      <c r="B137" t="n">
+        <v>9.94923</v>
+      </c>
+      <c r="C137" t="n">
+        <v>12.44364110656686</v>
+      </c>
+      <c r="D137" t="n">
+        <v>14.7936682809096</v>
+      </c>
+      <c r="E137" t="n">
+        <v>163.8876273488021</v>
+      </c>
+      <c r="F137" t="n">
+        <v>171.792233651628</v>
+      </c>
+      <c r="G137" t="n">
+        <v>176.136707751836</v>
+      </c>
+      <c r="H137" t="n">
+        <v>170.7824282111847</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="1" t="n">
+        <v>136</v>
+      </c>
+      <c r="B138" t="n">
+        <v>10.014161</v>
+      </c>
+      <c r="C138" t="n">
+        <v>12.67675324310277</v>
+      </c>
+      <c r="D138" t="n">
+        <v>14.66489149011127</v>
+      </c>
+      <c r="E138" t="n">
+        <v>163.7805102642125</v>
+      </c>
+      <c r="F138" t="n">
+        <v>171.6350697315245</v>
+      </c>
+      <c r="G138" t="n">
+        <v>176.024224720407</v>
+      </c>
+      <c r="H138" t="n">
+        <v>171.1068097671507</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="1" t="n">
+        <v>137</v>
+      </c>
+      <c r="B139" t="n">
+        <v>10.087382</v>
+      </c>
+      <c r="C139" t="n">
+        <v>12.76177463676305</v>
+      </c>
+      <c r="D139" t="n">
+        <v>14.53208553988186</v>
+      </c>
+      <c r="E139" t="n">
+        <v>163.8629208980431</v>
+      </c>
+      <c r="F139" t="n">
+        <v>171.5929984199288</v>
+      </c>
+      <c r="G139" t="n">
+        <v>175.9373990843725</v>
+      </c>
+      <c r="H139" t="n">
+        <v>171.1567632121252</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="1" t="n">
+        <v>138</v>
+      </c>
+      <c r="B140" t="n">
+        <v>10.152127</v>
+      </c>
+      <c r="C140" t="n">
+        <v>11.88676839349192</v>
+      </c>
+      <c r="D140" t="n">
+        <v>14.44859846262778</v>
+      </c>
+      <c r="E140" t="n">
+        <v>165.4279334389535</v>
+      </c>
+      <c r="F140" t="n">
+        <v>172.4383328701567</v>
+      </c>
+      <c r="G140" t="n">
+        <v>176.4902402755388</v>
+      </c>
+      <c r="H140" t="n">
+        <v>170.8006610876371</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="1" t="n">
+        <v>139</v>
+      </c>
+      <c r="B141" t="n">
+        <v>10.221851</v>
+      </c>
+      <c r="C141" t="n">
+        <v>11.95173176544464</v>
+      </c>
+      <c r="D141" t="n">
+        <v>14.43455009876413</v>
+      </c>
+      <c r="E141" t="n">
+        <v>165.3544056462769</v>
+      </c>
+      <c r="F141" t="n">
+        <v>172.5685311119018</v>
+      </c>
+      <c r="G141" t="n">
+        <v>176.3031343230216</v>
+      </c>
+      <c r="H141" t="n">
+        <v>170.76559298351</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="1" t="n">
+        <v>140</v>
+      </c>
+      <c r="B142" t="n">
+        <v>10.302395</v>
+      </c>
+      <c r="C142" t="n">
+        <v>12.00315319994922</v>
+      </c>
+      <c r="D142" t="n">
+        <v>14.42733039769606</v>
+      </c>
+      <c r="E142" t="n">
+        <v>165.3393026781102</v>
+      </c>
+      <c r="F142" t="n">
+        <v>172.6176918991744</v>
+      </c>
+      <c r="G142" t="n">
+        <v>176.2580058553857</v>
+      </c>
+      <c r="H142" t="n">
+        <v>170.7131418344673</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="1" t="n">
+        <v>141</v>
+      </c>
+      <c r="B143" t="n">
+        <v>10.36541</v>
+      </c>
+      <c r="C143" t="n">
+        <v>11.53087051193947</v>
+      </c>
+      <c r="D143" t="n">
+        <v>14.46932414530249</v>
+      </c>
+      <c r="E143" t="n">
+        <v>165.3687286938881</v>
+      </c>
+      <c r="F143" t="n">
+        <v>173.1090631224987</v>
+      </c>
+      <c r="G143" t="n">
+        <v>176.0498903610572</v>
+      </c>
+      <c r="H143" t="n">
+        <v>170.2569767732282</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="1" t="n">
+        <v>142</v>
+      </c>
+      <c r="B144" t="n">
+        <v>10.44118</v>
+      </c>
+      <c r="C144" t="n">
+        <v>11.65524941238687</v>
+      </c>
+      <c r="D144" t="n">
+        <v>14.46168282609911</v>
+      </c>
+      <c r="E144" t="n">
+        <v>165.2788396298223</v>
+      </c>
+      <c r="F144" t="n">
+        <v>173.068622284295</v>
+      </c>
+      <c r="G144" t="n">
+        <v>176.2068507996538</v>
+      </c>
+      <c r="H144" t="n">
+        <v>170.3196643892913</v>
       </c>
     </row>
   </sheetData>

</xml_diff>